<commit_message>
Extruder Report: Mylenes Report was completed
</commit_message>
<xml_diff>
--- a/app/views/extruder_form/records/extruder_report_format.xlsx
+++ b/app/views/extruder_form/records/extruder_report_format.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\MBPI-Projects\DEPLOYMENT-MixerExtruder-Project\app\views\extruder_form\records\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7F5841F-D1F9-4A6A-80CD-916BBF3B8F58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56E06533-A58B-463C-AD93-BD29D488DD19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A8C50F24-49C3-4045-93FC-1EB156652CF7}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="34">
   <si>
     <t xml:space="preserve">MC# </t>
   </si>
@@ -78,9 +78,6 @@
     <t>%</t>
   </si>
   <si>
-    <t>Loss %</t>
-  </si>
-  <si>
     <t/>
   </si>
   <si>
@@ -102,9 +99,6 @@
     <t>Lot #</t>
   </si>
   <si>
-    <t>Total</t>
-  </si>
-  <si>
     <t>Purging to :</t>
   </si>
   <si>
@@ -133,6 +127,15 @@
   </si>
   <si>
     <t xml:space="preserve">Extruder Machine No. </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> %</t>
+  </si>
+  <si>
+    <t>Total Input</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total   </t>
   </si>
 </sst>
 </file>
@@ -201,7 +204,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -214,8 +217,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="47">
+  <borders count="41">
     <border>
       <left/>
       <right/>
@@ -378,15 +387,6 @@
     </border>
     <border>
       <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right/>
       <top/>
       <bottom style="medium">
@@ -605,112 +605,9 @@
     <border>
       <left/>
       <right style="medium">
-        <color indexed="8"/>
+        <color auto="1"/>
       </right>
       <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="8"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="8"/>
-      </left>
-      <right style="thin">
-        <color indexed="8"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="8"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="8"/>
-      </left>
-      <right style="thin">
-        <color indexed="8"/>
-      </right>
-      <top style="thin">
-        <color indexed="8"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="8"/>
-      </right>
-      <top style="thin">
-        <color indexed="8"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -743,6 +640,54 @@
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="8"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -750,7 +695,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="95">
+  <cellXfs count="96">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -767,151 +712,182 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="4" fontId="3" fillId="2" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="3" fillId="2" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="31" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="4" fillId="0" borderId="33" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="34" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="35" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="35" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="3" fillId="0" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="3" fillId="3" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="21" fontId="3" fillId="0" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="3" fillId="2" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="3" fillId="0" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="3" fillId="2" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="4" fillId="0" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="39" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="40" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="40" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="3" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="4" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="30" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="3" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="3" fillId="0" borderId="31" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="31" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="34" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="3" fillId="0" borderId="35" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="21" fontId="4" fillId="0" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="32" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="41" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="42" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="26" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="43" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="4" fillId="0" borderId="41" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="4" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="46" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="44" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="45" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="45" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -933,74 +909,48 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="4" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="4" fillId="0" borderId="36" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="38" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="26" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="35" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="31" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1321,8 +1271,9 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="2.28515625" customWidth="1"/>
-    <col min="5" max="5" width="13.28515625" customWidth="1"/>
-    <col min="13" max="13" width="11.5703125" customWidth="1"/>
+    <col min="5" max="5" width="14.140625" customWidth="1"/>
+    <col min="10" max="10" width="12.85546875" customWidth="1"/>
+    <col min="13" max="13" width="18.42578125" customWidth="1"/>
     <col min="14" max="14" width="13.28515625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1333,13 +1284,13 @@
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
-      <c r="F5" s="57" t="s">
-        <v>32</v>
-      </c>
-      <c r="G5" s="58"/>
-      <c r="H5" s="58"/>
-      <c r="I5" s="58"/>
-      <c r="J5" s="59"/>
+      <c r="F5" s="68" t="s">
+        <v>30</v>
+      </c>
+      <c r="G5" s="69"/>
+      <c r="H5" s="69"/>
+      <c r="I5" s="69"/>
+      <c r="J5" s="70"/>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
@@ -1367,16 +1318,16 @@
       <c r="B7" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C7" s="60" t="s">
+      <c r="C7" s="71" t="s">
         <v>2</v>
       </c>
-      <c r="D7" s="61"/>
-      <c r="E7" s="62"/>
+      <c r="D7" s="72"/>
+      <c r="E7" s="73"/>
       <c r="F7" s="3" t="s">
         <v>3</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>4</v>
+        <v>32</v>
       </c>
       <c r="H7" s="3" t="s">
         <v>5</v>
@@ -1390,491 +1341,448 @@
       <c r="K7" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="L7" s="3"/>
+      <c r="L7" s="3" t="s">
+        <v>18</v>
+      </c>
       <c r="M7" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="N7" s="5"/>
+      <c r="N7" s="5" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="8" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="63"/>
-      <c r="B8" s="65"/>
-      <c r="C8" s="67"/>
-      <c r="D8" s="56"/>
-      <c r="E8" s="68"/>
-      <c r="F8" s="71"/>
-      <c r="G8" s="6" t="s">
+      <c r="A8" s="74"/>
+      <c r="B8" s="76"/>
+      <c r="C8" s="78"/>
+      <c r="D8" s="79"/>
+      <c r="E8" s="80"/>
+      <c r="F8" s="83"/>
+      <c r="G8" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="H8" s="6" t="s">
+      <c r="H8" s="34" t="s">
         <v>11</v>
       </c>
-      <c r="I8" s="6" t="s">
+      <c r="I8" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="J8" s="6" t="s">
+      <c r="J8" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="K8" s="6" t="s">
+      <c r="K8" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="L8" s="6" t="s">
+      <c r="L8" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="M8" s="6" t="s">
+      <c r="M8" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="N8" s="7" t="s">
+      <c r="N8" s="21" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="75"/>
+      <c r="B9" s="77"/>
+      <c r="C9" s="81"/>
+      <c r="D9" s="82"/>
+      <c r="E9" s="77"/>
+      <c r="F9" s="81"/>
+      <c r="G9" s="6"/>
+      <c r="H9" s="6"/>
+      <c r="I9" s="6"/>
+      <c r="J9" s="32"/>
+      <c r="K9" s="6"/>
+      <c r="L9" s="6"/>
+      <c r="M9" s="6"/>
+      <c r="N9" s="7"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10" s="8"/>
+      <c r="B10" s="34"/>
+      <c r="C10" s="34"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="34"/>
+      <c r="G10" s="34"/>
+      <c r="H10" s="35"/>
+      <c r="I10" s="34"/>
+      <c r="J10" s="34" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="9" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="64"/>
-      <c r="B9" s="66"/>
-      <c r="C9" s="69"/>
-      <c r="D9" s="70"/>
-      <c r="E9" s="66"/>
-      <c r="F9" s="69"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="8"/>
-      <c r="I9" s="8"/>
-      <c r="J9" s="9"/>
-      <c r="K9" s="8"/>
-      <c r="L9" s="8"/>
-      <c r="M9" s="8"/>
-      <c r="N9" s="10"/>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A10" s="11"/>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="12"/>
-      <c r="E10" s="12"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="13"/>
-      <c r="I10" s="6"/>
-      <c r="J10" s="6" t="s">
+      <c r="K10" s="34"/>
+      <c r="L10" s="34"/>
+      <c r="M10" s="34"/>
+      <c r="N10" s="36"/>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11" s="84" t="s">
         <v>15</v>
       </c>
-      <c r="K10" s="6"/>
-      <c r="L10" s="6"/>
-      <c r="M10" s="6"/>
-      <c r="N10" s="14"/>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="72" t="s">
+      <c r="B11" s="64"/>
+      <c r="C11" s="65"/>
+      <c r="D11" s="85" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="52"/>
-      <c r="C11" s="53"/>
-      <c r="D11" s="73" t="s">
+      <c r="E11" s="56"/>
+      <c r="F11" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="E11" s="55"/>
-      <c r="F11" s="15" t="s">
+      <c r="G11" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="G11" s="15" t="s">
+      <c r="H11" s="34"/>
+      <c r="I11" s="37" t="s">
         <v>19</v>
       </c>
-      <c r="H11" s="6"/>
-      <c r="I11" s="16" t="s">
+      <c r="J11" s="34"/>
+      <c r="K11" s="34"/>
+      <c r="L11" s="34"/>
+      <c r="M11" s="37" t="s">
         <v>20</v>
       </c>
-      <c r="J11" s="6"/>
-      <c r="K11" s="6"/>
-      <c r="L11" s="6"/>
-      <c r="M11" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="N11" s="14"/>
+      <c r="N11" s="21" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A12" s="74"/>
-      <c r="B12" s="52"/>
-      <c r="C12" s="53"/>
-      <c r="D12" s="54"/>
-      <c r="E12" s="55"/>
-      <c r="F12" s="17">
-        <v>0.17708333333333329</v>
-      </c>
-      <c r="G12" s="18">
-        <v>255.35</v>
-      </c>
-      <c r="H12" s="6"/>
-      <c r="I12" s="91"/>
-      <c r="J12" s="92"/>
-      <c r="K12" s="19"/>
-      <c r="L12" s="6"/>
-      <c r="M12" s="20"/>
-      <c r="N12" s="21"/>
+      <c r="A12" s="86"/>
+      <c r="B12" s="64"/>
+      <c r="C12" s="65"/>
+      <c r="D12" s="55"/>
+      <c r="E12" s="56"/>
+      <c r="F12" s="11"/>
+      <c r="G12" s="12"/>
+      <c r="H12" s="34"/>
+      <c r="I12" s="87"/>
+      <c r="J12" s="88"/>
+      <c r="K12" s="13"/>
+      <c r="L12" s="34"/>
+      <c r="M12" s="14"/>
+      <c r="N12" s="15"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A13" s="51"/>
-      <c r="B13" s="52"/>
-      <c r="C13" s="53"/>
-      <c r="D13" s="54"/>
-      <c r="E13" s="55"/>
-      <c r="F13" s="22"/>
-      <c r="G13" s="23"/>
-      <c r="H13" s="24"/>
-      <c r="I13" s="93"/>
-      <c r="J13" s="94"/>
-      <c r="K13" s="25"/>
-      <c r="L13" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="M13" s="26"/>
-      <c r="N13" s="14"/>
+      <c r="A13" s="66"/>
+      <c r="B13" s="64"/>
+      <c r="C13" s="65"/>
+      <c r="D13" s="55"/>
+      <c r="E13" s="56"/>
+      <c r="F13" s="16"/>
+      <c r="G13" s="17"/>
+      <c r="H13" s="38"/>
+      <c r="I13" s="57"/>
+      <c r="J13" s="58"/>
+      <c r="K13" s="18"/>
+      <c r="L13" s="34" t="s">
+        <v>14</v>
+      </c>
+      <c r="M13" s="19"/>
+      <c r="N13" s="36"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" s="51"/>
-      <c r="B14" s="52"/>
-      <c r="C14" s="53"/>
-      <c r="D14" s="54"/>
-      <c r="E14" s="55"/>
-      <c r="F14" s="22"/>
-      <c r="G14" s="23"/>
-      <c r="H14" s="27"/>
-      <c r="I14" s="93"/>
-      <c r="J14" s="94"/>
-      <c r="K14" s="25"/>
-      <c r="L14" s="6"/>
-      <c r="M14" s="26"/>
-      <c r="N14" s="14"/>
+      <c r="A14" s="66"/>
+      <c r="B14" s="64"/>
+      <c r="C14" s="65"/>
+      <c r="D14" s="55"/>
+      <c r="E14" s="56"/>
+      <c r="F14" s="16"/>
+      <c r="G14" s="17"/>
+      <c r="H14" s="39"/>
+      <c r="I14" s="57"/>
+      <c r="J14" s="58"/>
+      <c r="K14" s="18"/>
+      <c r="L14" s="34"/>
+      <c r="M14" s="19"/>
+      <c r="N14" s="36"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" s="51"/>
-      <c r="B15" s="52"/>
-      <c r="C15" s="53"/>
-      <c r="D15" s="54"/>
-      <c r="E15" s="55"/>
-      <c r="F15" s="22"/>
-      <c r="G15" s="23"/>
-      <c r="H15" s="27"/>
-      <c r="I15" s="93"/>
-      <c r="J15" s="94"/>
-      <c r="K15" s="25"/>
-      <c r="L15" s="6"/>
-      <c r="M15" s="26"/>
-      <c r="N15" s="14"/>
+      <c r="A15" s="66"/>
+      <c r="B15" s="64"/>
+      <c r="C15" s="65"/>
+      <c r="D15" s="55"/>
+      <c r="E15" s="56"/>
+      <c r="F15" s="16"/>
+      <c r="G15" s="17"/>
+      <c r="H15" s="39"/>
+      <c r="I15" s="57"/>
+      <c r="J15" s="58"/>
+      <c r="K15" s="18"/>
+      <c r="L15" s="34"/>
+      <c r="M15" s="19"/>
+      <c r="N15" s="36"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A16" s="51"/>
-      <c r="B16" s="52"/>
-      <c r="C16" s="53"/>
-      <c r="D16" s="75"/>
-      <c r="E16" s="55"/>
-      <c r="F16" s="22"/>
-      <c r="G16" s="23"/>
-      <c r="H16" s="27"/>
-      <c r="I16" s="93"/>
-      <c r="J16" s="94"/>
-      <c r="K16" s="25"/>
-      <c r="L16" s="6"/>
-      <c r="M16" s="26"/>
-      <c r="N16" s="14"/>
+      <c r="A16" s="66"/>
+      <c r="B16" s="64"/>
+      <c r="C16" s="65"/>
+      <c r="D16" s="67"/>
+      <c r="E16" s="56"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="17"/>
+      <c r="H16" s="39"/>
+      <c r="I16" s="57"/>
+      <c r="J16" s="58"/>
+      <c r="K16" s="18"/>
+      <c r="L16" s="34"/>
+      <c r="M16" s="19"/>
+      <c r="N16" s="36"/>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A17" s="51"/>
-      <c r="B17" s="52"/>
-      <c r="C17" s="53"/>
-      <c r="D17" s="75"/>
-      <c r="E17" s="55"/>
-      <c r="F17" s="22"/>
-      <c r="G17" s="23"/>
-      <c r="H17" s="27"/>
-      <c r="I17" s="93"/>
-      <c r="J17" s="94"/>
-      <c r="K17" s="25"/>
-      <c r="L17" s="6"/>
-      <c r="M17" s="26"/>
-      <c r="N17" s="14"/>
+      <c r="A17" s="66"/>
+      <c r="B17" s="64"/>
+      <c r="C17" s="65"/>
+      <c r="D17" s="67"/>
+      <c r="E17" s="56"/>
+      <c r="F17" s="16"/>
+      <c r="G17" s="17"/>
+      <c r="H17" s="39"/>
+      <c r="I17" s="57"/>
+      <c r="J17" s="58"/>
+      <c r="K17" s="18"/>
+      <c r="L17" s="34"/>
+      <c r="M17" s="19"/>
+      <c r="N17" s="36"/>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A18" s="51"/>
-      <c r="B18" s="52"/>
-      <c r="C18" s="53"/>
-      <c r="D18" s="54"/>
-      <c r="E18" s="55"/>
-      <c r="F18" s="22"/>
-      <c r="G18" s="23"/>
-      <c r="H18" s="27"/>
-      <c r="I18" s="93"/>
-      <c r="J18" s="94"/>
-      <c r="K18" s="25"/>
-      <c r="L18" s="6"/>
-      <c r="M18" s="26"/>
-      <c r="N18" s="14"/>
+      <c r="A18" s="66"/>
+      <c r="B18" s="64"/>
+      <c r="C18" s="65"/>
+      <c r="D18" s="55"/>
+      <c r="E18" s="56"/>
+      <c r="F18" s="16"/>
+      <c r="G18" s="17"/>
+      <c r="H18" s="39"/>
+      <c r="I18" s="57"/>
+      <c r="J18" s="58"/>
+      <c r="K18" s="18"/>
+      <c r="L18" s="34"/>
+      <c r="M18" s="19"/>
+      <c r="N18" s="36"/>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A19" s="76"/>
-      <c r="B19" s="52"/>
-      <c r="C19" s="53"/>
-      <c r="D19" s="54"/>
-      <c r="E19" s="55"/>
-      <c r="F19" s="22"/>
-      <c r="G19" s="23"/>
-      <c r="H19" s="28"/>
-      <c r="I19" s="93"/>
-      <c r="J19" s="94"/>
-      <c r="K19" s="25"/>
-      <c r="L19" s="29"/>
-      <c r="M19" s="26"/>
-      <c r="N19" s="30"/>
+      <c r="A19" s="53"/>
+      <c r="B19" s="64"/>
+      <c r="C19" s="65"/>
+      <c r="D19" s="55"/>
+      <c r="E19" s="56"/>
+      <c r="F19" s="16"/>
+      <c r="G19" s="17"/>
+      <c r="H19" s="40"/>
+      <c r="I19" s="57"/>
+      <c r="J19" s="58"/>
+      <c r="K19" s="18"/>
+      <c r="L19" s="41"/>
+      <c r="M19" s="19"/>
+      <c r="N19" s="36"/>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A20" s="76"/>
-      <c r="B20" s="52"/>
-      <c r="C20" s="53"/>
-      <c r="D20" s="54"/>
-      <c r="E20" s="55"/>
-      <c r="F20" s="22"/>
-      <c r="G20" s="23"/>
-      <c r="H20" s="28"/>
-      <c r="I20" s="93"/>
-      <c r="J20" s="94"/>
-      <c r="K20" s="25"/>
-      <c r="L20" s="29"/>
-      <c r="M20" s="26"/>
-      <c r="N20" s="30"/>
+      <c r="A20" s="53"/>
+      <c r="B20" s="64"/>
+      <c r="C20" s="65"/>
+      <c r="D20" s="55"/>
+      <c r="E20" s="56"/>
+      <c r="F20" s="16"/>
+      <c r="G20" s="17"/>
+      <c r="H20" s="40"/>
+      <c r="I20" s="57"/>
+      <c r="J20" s="58"/>
+      <c r="K20" s="18"/>
+      <c r="L20" s="41"/>
+      <c r="M20" s="19"/>
+      <c r="N20" s="36"/>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A21" s="76"/>
-      <c r="B21" s="52"/>
-      <c r="C21" s="53"/>
-      <c r="D21" s="54"/>
-      <c r="E21" s="55"/>
-      <c r="F21" s="22"/>
-      <c r="G21" s="23"/>
-      <c r="H21" s="28"/>
-      <c r="I21" s="93"/>
-      <c r="J21" s="94"/>
-      <c r="K21" s="25"/>
-      <c r="L21" s="29"/>
-      <c r="M21" s="26"/>
-      <c r="N21" s="30"/>
+      <c r="A21" s="53"/>
+      <c r="B21" s="64"/>
+      <c r="C21" s="65"/>
+      <c r="D21" s="55"/>
+      <c r="E21" s="56"/>
+      <c r="F21" s="16"/>
+      <c r="G21" s="17"/>
+      <c r="H21" s="40"/>
+      <c r="I21" s="57"/>
+      <c r="J21" s="58"/>
+      <c r="K21" s="18"/>
+      <c r="L21" s="41"/>
+      <c r="M21" s="19"/>
+      <c r="N21" s="36"/>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A22" s="76"/>
-      <c r="B22" s="52"/>
-      <c r="C22" s="53"/>
-      <c r="D22" s="54"/>
-      <c r="E22" s="55"/>
-      <c r="F22" s="22"/>
-      <c r="G22" s="23"/>
-      <c r="H22" s="28"/>
-      <c r="I22" s="93"/>
-      <c r="J22" s="94"/>
-      <c r="K22" s="25"/>
-      <c r="L22" s="29"/>
-      <c r="M22" s="26"/>
-      <c r="N22" s="30"/>
+      <c r="A22" s="53"/>
+      <c r="B22" s="64"/>
+      <c r="C22" s="65"/>
+      <c r="D22" s="55"/>
+      <c r="E22" s="56"/>
+      <c r="F22" s="16"/>
+      <c r="G22" s="17"/>
+      <c r="H22" s="40"/>
+      <c r="I22" s="57"/>
+      <c r="J22" s="58"/>
+      <c r="K22" s="18"/>
+      <c r="L22" s="41"/>
+      <c r="M22" s="19"/>
+      <c r="N22" s="36"/>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A23" s="76"/>
-      <c r="B23" s="52"/>
-      <c r="C23" s="53"/>
-      <c r="D23" s="54"/>
-      <c r="E23" s="55"/>
-      <c r="F23" s="22"/>
-      <c r="G23" s="23"/>
-      <c r="H23" s="28"/>
-      <c r="I23" s="93"/>
-      <c r="J23" s="94"/>
-      <c r="K23" s="25"/>
-      <c r="L23" s="29"/>
-      <c r="M23" s="26"/>
-      <c r="N23" s="30"/>
+      <c r="A23" s="53"/>
+      <c r="B23" s="64"/>
+      <c r="C23" s="65"/>
+      <c r="D23" s="55"/>
+      <c r="E23" s="56"/>
+      <c r="F23" s="16"/>
+      <c r="G23" s="17"/>
+      <c r="H23" s="40"/>
+      <c r="I23" s="57"/>
+      <c r="J23" s="58"/>
+      <c r="K23" s="18"/>
+      <c r="L23" s="41"/>
+      <c r="M23" s="19"/>
+      <c r="N23" s="36"/>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A24" s="76"/>
-      <c r="B24" s="52"/>
-      <c r="C24" s="53"/>
-      <c r="D24" s="54"/>
-      <c r="E24" s="55"/>
-      <c r="F24" s="20"/>
-      <c r="G24" s="23"/>
-      <c r="H24" s="28"/>
-      <c r="I24" s="93"/>
-      <c r="J24" s="94"/>
-      <c r="K24" s="25"/>
-      <c r="L24" s="29"/>
-      <c r="M24" s="26"/>
-      <c r="N24" s="30"/>
-    </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A25" s="31" t="s">
-        <v>22</v>
-      </c>
-      <c r="B25" s="81"/>
-      <c r="C25" s="82"/>
-      <c r="D25" s="83"/>
-      <c r="E25" s="84"/>
-      <c r="F25" s="32">
-        <v>0.17708333333333329</v>
-      </c>
-      <c r="G25" s="23">
+      <c r="A24" s="53"/>
+      <c r="B24" s="54"/>
+      <c r="C24" s="54"/>
+      <c r="D24" s="55"/>
+      <c r="E24" s="56"/>
+      <c r="F24" s="14"/>
+      <c r="G24" s="17"/>
+      <c r="H24" s="40"/>
+      <c r="I24" s="57"/>
+      <c r="J24" s="58"/>
+      <c r="K24" s="18"/>
+      <c r="L24" s="41"/>
+      <c r="M24" s="19"/>
+      <c r="N24" s="36"/>
+    </row>
+    <row r="25" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="61" t="s">
+        <v>33</v>
+      </c>
+      <c r="B25" s="62"/>
+      <c r="C25" s="62"/>
+      <c r="D25" s="62"/>
+      <c r="E25" s="63"/>
+      <c r="F25" s="33"/>
+      <c r="G25" s="31">
         <f>SUM(G12:G24)</f>
-        <v>255.35</v>
-      </c>
-      <c r="H25" s="6"/>
-      <c r="I25" s="33" t="s">
-        <v>22</v>
-      </c>
-      <c r="J25" s="29"/>
-      <c r="K25" s="34">
+        <v>0</v>
+      </c>
+      <c r="H25" s="34"/>
+      <c r="I25" s="42" t="s">
+        <v>32</v>
+      </c>
+      <c r="J25" s="43"/>
+      <c r="K25" s="44">
         <f>SUM(K12:K24)</f>
         <v>0</v>
       </c>
-      <c r="L25" s="29"/>
-      <c r="M25" s="26"/>
-      <c r="N25" s="30"/>
+      <c r="L25" s="41"/>
+      <c r="M25" s="19"/>
+      <c r="N25" s="36"/>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A26" s="35" t="s">
+      <c r="A26" s="45" t="s">
+        <v>21</v>
+      </c>
+      <c r="B26" s="59"/>
+      <c r="C26" s="59"/>
+      <c r="D26" s="59"/>
+      <c r="E26" s="46" t="s">
+        <v>22</v>
+      </c>
+      <c r="F26" s="47" t="s">
         <v>23</v>
       </c>
-      <c r="B26" s="85"/>
-      <c r="C26" s="85"/>
-      <c r="D26" s="85"/>
-      <c r="E26" s="36" t="s">
+      <c r="G26" s="89"/>
+      <c r="H26" s="89"/>
+      <c r="I26" s="89"/>
+      <c r="J26" s="89"/>
+      <c r="K26" s="48"/>
+      <c r="L26" s="48"/>
+      <c r="M26" s="3"/>
+      <c r="N26" s="5"/>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A27" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="F26" s="37" t="s">
+      <c r="B27" s="60"/>
+      <c r="C27" s="60"/>
+      <c r="D27" s="60"/>
+      <c r="E27" s="22"/>
+      <c r="F27" s="23"/>
+      <c r="G27" s="90"/>
+      <c r="H27" s="90"/>
+      <c r="I27" s="90"/>
+      <c r="J27" s="90"/>
+      <c r="K27" s="40"/>
+      <c r="L27" s="40"/>
+      <c r="M27" s="34"/>
+      <c r="N27" s="36"/>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A28" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="G26" s="86"/>
-      <c r="H26" s="86"/>
-      <c r="I26" s="86"/>
-      <c r="J26" s="86"/>
-      <c r="K26" s="38"/>
-      <c r="L26" s="38"/>
-      <c r="M26" s="39"/>
-      <c r="N26" s="40"/>
-    </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A27" s="35" t="s">
+      <c r="B28" s="94"/>
+      <c r="C28" s="94"/>
+      <c r="D28" s="94"/>
+      <c r="E28" s="95"/>
+      <c r="F28" s="23"/>
+      <c r="G28" s="90"/>
+      <c r="H28" s="90"/>
+      <c r="I28" s="90"/>
+      <c r="J28" s="90"/>
+      <c r="K28" s="40"/>
+      <c r="L28" s="37" t="s">
         <v>26</v>
       </c>
-      <c r="B27" s="88"/>
-      <c r="C27" s="88"/>
-      <c r="D27" s="88"/>
-      <c r="E27" s="41"/>
-      <c r="F27" s="42"/>
-      <c r="G27" s="87"/>
-      <c r="H27" s="87"/>
-      <c r="I27" s="87"/>
-      <c r="J27" s="87"/>
-      <c r="K27" s="28"/>
-      <c r="L27" s="28"/>
-      <c r="M27" s="6"/>
-      <c r="N27" s="14"/>
-    </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A28" s="35" t="s">
+      <c r="M28" s="92"/>
+      <c r="N28" s="93"/>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A29" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="B28" s="89"/>
-      <c r="C28" s="89"/>
-      <c r="D28" s="89"/>
-      <c r="E28" s="90"/>
-      <c r="F28" s="42"/>
-      <c r="G28" s="87"/>
-      <c r="H28" s="87"/>
-      <c r="I28" s="87"/>
-      <c r="J28" s="87"/>
-      <c r="K28" s="28"/>
-      <c r="L28" s="16" t="s">
+      <c r="B29" s="51"/>
+      <c r="C29" s="51"/>
+      <c r="D29" s="51"/>
+      <c r="E29" s="22"/>
+      <c r="F29" s="23"/>
+      <c r="G29" s="90"/>
+      <c r="H29" s="90"/>
+      <c r="I29" s="90"/>
+      <c r="J29" s="90"/>
+      <c r="K29" s="40"/>
+      <c r="L29" s="37" t="s">
         <v>28</v>
       </c>
-      <c r="M28" s="77"/>
-      <c r="N28" s="78"/>
-    </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A29" s="35" t="s">
+      <c r="M29" s="49"/>
+      <c r="N29" s="50"/>
+    </row>
+    <row r="30" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="B29" s="79"/>
-      <c r="C29" s="79"/>
-      <c r="D29" s="79"/>
-      <c r="E29" s="43"/>
-      <c r="F29" s="42"/>
-      <c r="G29" s="87"/>
-      <c r="H29" s="87"/>
-      <c r="I29" s="87"/>
-      <c r="J29" s="87"/>
-      <c r="K29" s="28"/>
-      <c r="L29" s="16" t="s">
-        <v>30</v>
-      </c>
-      <c r="M29" s="77"/>
-      <c r="N29" s="78"/>
-    </row>
-    <row r="30" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="44" t="s">
-        <v>31</v>
-      </c>
-      <c r="B30" s="80"/>
-      <c r="C30" s="80"/>
-      <c r="D30" s="80"/>
-      <c r="E30" s="46"/>
-      <c r="F30" s="47"/>
-      <c r="G30" s="48"/>
-      <c r="H30" s="49"/>
-      <c r="I30" s="49"/>
-      <c r="J30" s="49"/>
-      <c r="K30" s="48"/>
-      <c r="L30" s="49"/>
-      <c r="M30" s="45"/>
-      <c r="N30" s="50"/>
+      <c r="B30" s="52"/>
+      <c r="C30" s="52"/>
+      <c r="D30" s="52"/>
+      <c r="E30" s="26"/>
+      <c r="F30" s="27"/>
+      <c r="G30" s="91"/>
+      <c r="H30" s="91"/>
+      <c r="I30" s="91"/>
+      <c r="J30" s="91"/>
+      <c r="K30" s="28"/>
+      <c r="L30" s="29"/>
+      <c r="M30" s="25"/>
+      <c r="N30" s="30"/>
     </row>
   </sheetData>
-  <mergeCells count="57">
-    <mergeCell ref="M28:N28"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="M29:N29"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="A24:C24"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="I24:J24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="G26:J29"/>
-    <mergeCell ref="B27:D27"/>
-    <mergeCell ref="B28:E28"/>
-    <mergeCell ref="A22:C22"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="I22:J22"/>
-    <mergeCell ref="A23:C23"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="I23:J23"/>
-    <mergeCell ref="A20:C20"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="A21:C21"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="I21:J21"/>
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="I18:J18"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="D19:E19"/>
-    <mergeCell ref="I19:J19"/>
-    <mergeCell ref="A16:C16"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="I16:J16"/>
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="I17:J17"/>
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="I14:J14"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="I15:J15"/>
+  <mergeCells count="56">
     <mergeCell ref="A13:C13"/>
     <mergeCell ref="D13:E13"/>
     <mergeCell ref="I13:J13"/>
@@ -1889,7 +1797,50 @@
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="D12:E12"/>
     <mergeCell ref="I12:J12"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="I14:J14"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="I15:J15"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="I16:J16"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="I17:J17"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="D19:E19"/>
+    <mergeCell ref="I19:J19"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="I21:J21"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="I22:J22"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="I23:J23"/>
+    <mergeCell ref="M28:N28"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="M29:N29"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="I24:J24"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="B28:E28"/>
+    <mergeCell ref="G26:J30"/>
+    <mergeCell ref="A25:E25"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="5" scale="110" fitToWidth="0" orientation="landscape" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Extruder Form: Old records modification.
</commit_message>
<xml_diff>
--- a/app/views/extruder_form/records/extruder_report_format.xlsx
+++ b/app/views/extruder_form/records/extruder_report_format.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\MBPI-Projects\DEPLOYMENT-MixerExtruder-Project\app\views\extruder_form\records\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56E06533-A58B-463C-AD93-BD29D488DD19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1B4EF37-9518-4D8D-86FA-FF21016B686C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A8C50F24-49C3-4045-93FC-1EB156652CF7}"/>
   </bookViews>
@@ -695,7 +695,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="97">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -733,22 +733,13 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="4" fontId="4" fillId="0" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="31" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -826,9 +817,6 @@
     <xf numFmtId="4" fontId="4" fillId="0" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="39" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="40" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -841,13 +829,34 @@
     <xf numFmtId="168" fontId="3" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="4" fontId="3" fillId="0" borderId="39" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="26" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="31" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="28" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="33" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -870,6 +879,21 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="35" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="16" fontId="3" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -930,27 +954,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="35" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1284,13 +1287,13 @@
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
-      <c r="F5" s="68" t="s">
+      <c r="F5" s="76" t="s">
         <v>30</v>
       </c>
-      <c r="G5" s="69"/>
-      <c r="H5" s="69"/>
-      <c r="I5" s="69"/>
-      <c r="J5" s="70"/>
+      <c r="G5" s="77"/>
+      <c r="H5" s="77"/>
+      <c r="I5" s="77"/>
+      <c r="J5" s="78"/>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
@@ -1318,11 +1321,11 @@
       <c r="B7" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C7" s="71" t="s">
+      <c r="C7" s="79" t="s">
         <v>2</v>
       </c>
-      <c r="D7" s="72"/>
-      <c r="E7" s="73"/>
+      <c r="D7" s="80"/>
+      <c r="E7" s="81"/>
       <c r="F7" s="3" t="s">
         <v>3</v>
       </c>
@@ -1352,48 +1355,48 @@
       </c>
     </row>
     <row r="8" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="74"/>
-      <c r="B8" s="76"/>
-      <c r="C8" s="78"/>
-      <c r="D8" s="79"/>
-      <c r="E8" s="80"/>
-      <c r="F8" s="83"/>
-      <c r="G8" s="34" t="s">
+      <c r="A8" s="82"/>
+      <c r="B8" s="84"/>
+      <c r="C8" s="86"/>
+      <c r="D8" s="87"/>
+      <c r="E8" s="88"/>
+      <c r="F8" s="91"/>
+      <c r="G8" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="H8" s="34" t="s">
+      <c r="H8" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="I8" s="34" t="s">
+      <c r="I8" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="J8" s="34" t="s">
+      <c r="J8" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="K8" s="34" t="s">
+      <c r="K8" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="L8" s="34" t="s">
+      <c r="L8" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="M8" s="34" t="s">
+      <c r="M8" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="N8" s="21" t="s">
+      <c r="N8" s="18" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="75"/>
-      <c r="B9" s="77"/>
-      <c r="C9" s="81"/>
-      <c r="D9" s="82"/>
-      <c r="E9" s="77"/>
-      <c r="F9" s="81"/>
+      <c r="A9" s="83"/>
+      <c r="B9" s="85"/>
+      <c r="C9" s="89"/>
+      <c r="D9" s="90"/>
+      <c r="E9" s="85"/>
+      <c r="F9" s="89"/>
       <c r="G9" s="6"/>
       <c r="H9" s="6"/>
       <c r="I9" s="6"/>
-      <c r="J9" s="32"/>
+      <c r="J9" s="29"/>
       <c r="K9" s="6"/>
       <c r="L9" s="6"/>
       <c r="M9" s="6"/>
@@ -1401,385 +1404,385 @@
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="8"/>
-      <c r="B10" s="34"/>
-      <c r="C10" s="34"/>
+      <c r="B10" s="31"/>
+      <c r="C10" s="31"/>
       <c r="D10" s="9"/>
       <c r="E10" s="9"/>
-      <c r="F10" s="34"/>
-      <c r="G10" s="34"/>
-      <c r="H10" s="35"/>
-      <c r="I10" s="34"/>
-      <c r="J10" s="34" t="s">
+      <c r="F10" s="31"/>
+      <c r="G10" s="31"/>
+      <c r="H10" s="32"/>
+      <c r="I10" s="31"/>
+      <c r="J10" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="K10" s="34"/>
-      <c r="L10" s="34"/>
-      <c r="M10" s="34"/>
-      <c r="N10" s="36"/>
+      <c r="K10" s="31"/>
+      <c r="L10" s="31"/>
+      <c r="M10" s="31"/>
+      <c r="N10" s="33"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="84" t="s">
+      <c r="A11" s="92" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="64"/>
-      <c r="C11" s="65"/>
-      <c r="D11" s="85" t="s">
+      <c r="B11" s="72"/>
+      <c r="C11" s="73"/>
+      <c r="D11" s="93" t="s">
         <v>16</v>
       </c>
-      <c r="E11" s="56"/>
+      <c r="E11" s="59"/>
       <c r="F11" s="10" t="s">
         <v>17</v>
       </c>
       <c r="G11" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="H11" s="34"/>
-      <c r="I11" s="37" t="s">
+      <c r="H11" s="31"/>
+      <c r="I11" s="34" t="s">
         <v>19</v>
       </c>
-      <c r="J11" s="34"/>
-      <c r="K11" s="34"/>
-      <c r="L11" s="34"/>
-      <c r="M11" s="37" t="s">
+      <c r="J11" s="31"/>
+      <c r="K11" s="31"/>
+      <c r="L11" s="31"/>
+      <c r="M11" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="N11" s="21" t="s">
+      <c r="N11" s="18" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A12" s="86"/>
-      <c r="B12" s="64"/>
-      <c r="C12" s="65"/>
-      <c r="D12" s="55"/>
-      <c r="E12" s="56"/>
+      <c r="A12" s="94"/>
+      <c r="B12" s="72"/>
+      <c r="C12" s="73"/>
+      <c r="D12" s="58"/>
+      <c r="E12" s="59"/>
       <c r="F12" s="11"/>
       <c r="G12" s="12"/>
-      <c r="H12" s="34"/>
-      <c r="I12" s="87"/>
-      <c r="J12" s="88"/>
-      <c r="K12" s="13"/>
-      <c r="L12" s="34"/>
-      <c r="M12" s="14"/>
-      <c r="N12" s="15"/>
+      <c r="H12" s="31"/>
+      <c r="I12" s="95"/>
+      <c r="J12" s="96"/>
+      <c r="K12" s="46"/>
+      <c r="L12" s="31"/>
+      <c r="M12" s="13"/>
+      <c r="N12" s="48"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A13" s="66"/>
-      <c r="B13" s="64"/>
-      <c r="C13" s="65"/>
-      <c r="D13" s="55"/>
-      <c r="E13" s="56"/>
-      <c r="F13" s="16"/>
-      <c r="G13" s="17"/>
-      <c r="H13" s="38"/>
-      <c r="I13" s="57"/>
-      <c r="J13" s="58"/>
-      <c r="K13" s="18"/>
-      <c r="L13" s="34" t="s">
+      <c r="A13" s="74"/>
+      <c r="B13" s="72"/>
+      <c r="C13" s="73"/>
+      <c r="D13" s="58"/>
+      <c r="E13" s="59"/>
+      <c r="F13" s="14"/>
+      <c r="G13" s="15"/>
+      <c r="H13" s="35"/>
+      <c r="I13" s="60"/>
+      <c r="J13" s="61"/>
+      <c r="K13" s="47"/>
+      <c r="L13" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="M13" s="19"/>
-      <c r="N13" s="36"/>
+      <c r="M13" s="16"/>
+      <c r="N13" s="49"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" s="66"/>
-      <c r="B14" s="64"/>
-      <c r="C14" s="65"/>
-      <c r="D14" s="55"/>
-      <c r="E14" s="56"/>
-      <c r="F14" s="16"/>
-      <c r="G14" s="17"/>
-      <c r="H14" s="39"/>
-      <c r="I14" s="57"/>
-      <c r="J14" s="58"/>
-      <c r="K14" s="18"/>
-      <c r="L14" s="34"/>
-      <c r="M14" s="19"/>
-      <c r="N14" s="36"/>
+      <c r="A14" s="74"/>
+      <c r="B14" s="72"/>
+      <c r="C14" s="73"/>
+      <c r="D14" s="58"/>
+      <c r="E14" s="59"/>
+      <c r="F14" s="14"/>
+      <c r="G14" s="15"/>
+      <c r="H14" s="36"/>
+      <c r="I14" s="60"/>
+      <c r="J14" s="61"/>
+      <c r="K14" s="47"/>
+      <c r="L14" s="31"/>
+      <c r="M14" s="16"/>
+      <c r="N14" s="49"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" s="66"/>
-      <c r="B15" s="64"/>
-      <c r="C15" s="65"/>
-      <c r="D15" s="55"/>
-      <c r="E15" s="56"/>
-      <c r="F15" s="16"/>
-      <c r="G15" s="17"/>
-      <c r="H15" s="39"/>
-      <c r="I15" s="57"/>
-      <c r="J15" s="58"/>
-      <c r="K15" s="18"/>
-      <c r="L15" s="34"/>
-      <c r="M15" s="19"/>
-      <c r="N15" s="36"/>
+      <c r="A15" s="74"/>
+      <c r="B15" s="72"/>
+      <c r="C15" s="73"/>
+      <c r="D15" s="58"/>
+      <c r="E15" s="59"/>
+      <c r="F15" s="14"/>
+      <c r="G15" s="15"/>
+      <c r="H15" s="36"/>
+      <c r="I15" s="60"/>
+      <c r="J15" s="61"/>
+      <c r="K15" s="47"/>
+      <c r="L15" s="31"/>
+      <c r="M15" s="16"/>
+      <c r="N15" s="49"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A16" s="66"/>
-      <c r="B16" s="64"/>
-      <c r="C16" s="65"/>
-      <c r="D16" s="67"/>
-      <c r="E16" s="56"/>
-      <c r="F16" s="16"/>
-      <c r="G16" s="17"/>
-      <c r="H16" s="39"/>
-      <c r="I16" s="57"/>
-      <c r="J16" s="58"/>
-      <c r="K16" s="18"/>
-      <c r="L16" s="34"/>
-      <c r="M16" s="19"/>
-      <c r="N16" s="36"/>
+      <c r="A16" s="74"/>
+      <c r="B16" s="72"/>
+      <c r="C16" s="73"/>
+      <c r="D16" s="75"/>
+      <c r="E16" s="59"/>
+      <c r="F16" s="14"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="36"/>
+      <c r="I16" s="60"/>
+      <c r="J16" s="61"/>
+      <c r="K16" s="47"/>
+      <c r="L16" s="31"/>
+      <c r="M16" s="16"/>
+      <c r="N16" s="49"/>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A17" s="66"/>
-      <c r="B17" s="64"/>
-      <c r="C17" s="65"/>
-      <c r="D17" s="67"/>
-      <c r="E17" s="56"/>
-      <c r="F17" s="16"/>
-      <c r="G17" s="17"/>
-      <c r="H17" s="39"/>
-      <c r="I17" s="57"/>
-      <c r="J17" s="58"/>
-      <c r="K17" s="18"/>
-      <c r="L17" s="34"/>
-      <c r="M17" s="19"/>
-      <c r="N17" s="36"/>
+      <c r="A17" s="74"/>
+      <c r="B17" s="72"/>
+      <c r="C17" s="73"/>
+      <c r="D17" s="75"/>
+      <c r="E17" s="59"/>
+      <c r="F17" s="14"/>
+      <c r="G17" s="15"/>
+      <c r="H17" s="36"/>
+      <c r="I17" s="60"/>
+      <c r="J17" s="61"/>
+      <c r="K17" s="47"/>
+      <c r="L17" s="31"/>
+      <c r="M17" s="16"/>
+      <c r="N17" s="49"/>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A18" s="66"/>
-      <c r="B18" s="64"/>
-      <c r="C18" s="65"/>
-      <c r="D18" s="55"/>
-      <c r="E18" s="56"/>
-      <c r="F18" s="16"/>
-      <c r="G18" s="17"/>
-      <c r="H18" s="39"/>
-      <c r="I18" s="57"/>
-      <c r="J18" s="58"/>
-      <c r="K18" s="18"/>
-      <c r="L18" s="34"/>
-      <c r="M18" s="19"/>
-      <c r="N18" s="36"/>
+      <c r="A18" s="74"/>
+      <c r="B18" s="72"/>
+      <c r="C18" s="73"/>
+      <c r="D18" s="58"/>
+      <c r="E18" s="59"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="15"/>
+      <c r="H18" s="36"/>
+      <c r="I18" s="60"/>
+      <c r="J18" s="61"/>
+      <c r="K18" s="47"/>
+      <c r="L18" s="31"/>
+      <c r="M18" s="16"/>
+      <c r="N18" s="49"/>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A19" s="53"/>
-      <c r="B19" s="64"/>
-      <c r="C19" s="65"/>
-      <c r="D19" s="55"/>
-      <c r="E19" s="56"/>
-      <c r="F19" s="16"/>
-      <c r="G19" s="17"/>
-      <c r="H19" s="40"/>
-      <c r="I19" s="57"/>
-      <c r="J19" s="58"/>
-      <c r="K19" s="18"/>
-      <c r="L19" s="41"/>
-      <c r="M19" s="19"/>
-      <c r="N19" s="36"/>
+      <c r="A19" s="56"/>
+      <c r="B19" s="72"/>
+      <c r="C19" s="73"/>
+      <c r="D19" s="58"/>
+      <c r="E19" s="59"/>
+      <c r="F19" s="14"/>
+      <c r="G19" s="15"/>
+      <c r="H19" s="37"/>
+      <c r="I19" s="60"/>
+      <c r="J19" s="61"/>
+      <c r="K19" s="47"/>
+      <c r="L19" s="38"/>
+      <c r="M19" s="16"/>
+      <c r="N19" s="49"/>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A20" s="53"/>
-      <c r="B20" s="64"/>
-      <c r="C20" s="65"/>
-      <c r="D20" s="55"/>
-      <c r="E20" s="56"/>
-      <c r="F20" s="16"/>
-      <c r="G20" s="17"/>
-      <c r="H20" s="40"/>
-      <c r="I20" s="57"/>
-      <c r="J20" s="58"/>
-      <c r="K20" s="18"/>
-      <c r="L20" s="41"/>
-      <c r="M20" s="19"/>
-      <c r="N20" s="36"/>
+      <c r="A20" s="56"/>
+      <c r="B20" s="72"/>
+      <c r="C20" s="73"/>
+      <c r="D20" s="58"/>
+      <c r="E20" s="59"/>
+      <c r="F20" s="14"/>
+      <c r="G20" s="15"/>
+      <c r="H20" s="37"/>
+      <c r="I20" s="60"/>
+      <c r="J20" s="61"/>
+      <c r="K20" s="47"/>
+      <c r="L20" s="38"/>
+      <c r="M20" s="16"/>
+      <c r="N20" s="49"/>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A21" s="53"/>
-      <c r="B21" s="64"/>
-      <c r="C21" s="65"/>
-      <c r="D21" s="55"/>
-      <c r="E21" s="56"/>
-      <c r="F21" s="16"/>
-      <c r="G21" s="17"/>
-      <c r="H21" s="40"/>
-      <c r="I21" s="57"/>
-      <c r="J21" s="58"/>
-      <c r="K21" s="18"/>
-      <c r="L21" s="41"/>
-      <c r="M21" s="19"/>
-      <c r="N21" s="36"/>
+      <c r="A21" s="56"/>
+      <c r="B21" s="72"/>
+      <c r="C21" s="73"/>
+      <c r="D21" s="58"/>
+      <c r="E21" s="59"/>
+      <c r="F21" s="14"/>
+      <c r="G21" s="15"/>
+      <c r="H21" s="37"/>
+      <c r="I21" s="60"/>
+      <c r="J21" s="61"/>
+      <c r="K21" s="47"/>
+      <c r="L21" s="38"/>
+      <c r="M21" s="16"/>
+      <c r="N21" s="49"/>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A22" s="53"/>
-      <c r="B22" s="64"/>
-      <c r="C22" s="65"/>
-      <c r="D22" s="55"/>
-      <c r="E22" s="56"/>
-      <c r="F22" s="16"/>
-      <c r="G22" s="17"/>
-      <c r="H22" s="40"/>
-      <c r="I22" s="57"/>
-      <c r="J22" s="58"/>
-      <c r="K22" s="18"/>
-      <c r="L22" s="41"/>
-      <c r="M22" s="19"/>
-      <c r="N22" s="36"/>
+      <c r="A22" s="56"/>
+      <c r="B22" s="72"/>
+      <c r="C22" s="73"/>
+      <c r="D22" s="58"/>
+      <c r="E22" s="59"/>
+      <c r="F22" s="14"/>
+      <c r="G22" s="15"/>
+      <c r="H22" s="37"/>
+      <c r="I22" s="60"/>
+      <c r="J22" s="61"/>
+      <c r="K22" s="47"/>
+      <c r="L22" s="38"/>
+      <c r="M22" s="16"/>
+      <c r="N22" s="49"/>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A23" s="53"/>
-      <c r="B23" s="64"/>
-      <c r="C23" s="65"/>
-      <c r="D23" s="55"/>
-      <c r="E23" s="56"/>
-      <c r="F23" s="16"/>
-      <c r="G23" s="17"/>
-      <c r="H23" s="40"/>
-      <c r="I23" s="57"/>
-      <c r="J23" s="58"/>
-      <c r="K23" s="18"/>
-      <c r="L23" s="41"/>
-      <c r="M23" s="19"/>
-      <c r="N23" s="36"/>
+      <c r="A23" s="56"/>
+      <c r="B23" s="72"/>
+      <c r="C23" s="73"/>
+      <c r="D23" s="58"/>
+      <c r="E23" s="59"/>
+      <c r="F23" s="14"/>
+      <c r="G23" s="15"/>
+      <c r="H23" s="37"/>
+      <c r="I23" s="60"/>
+      <c r="J23" s="61"/>
+      <c r="K23" s="47"/>
+      <c r="L23" s="38"/>
+      <c r="M23" s="16"/>
+      <c r="N23" s="49"/>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A24" s="53"/>
-      <c r="B24" s="54"/>
-      <c r="C24" s="54"/>
-      <c r="D24" s="55"/>
-      <c r="E24" s="56"/>
-      <c r="F24" s="14"/>
-      <c r="G24" s="17"/>
-      <c r="H24" s="40"/>
-      <c r="I24" s="57"/>
-      <c r="J24" s="58"/>
-      <c r="K24" s="18"/>
-      <c r="L24" s="41"/>
-      <c r="M24" s="19"/>
-      <c r="N24" s="36"/>
+      <c r="A24" s="56"/>
+      <c r="B24" s="57"/>
+      <c r="C24" s="57"/>
+      <c r="D24" s="58"/>
+      <c r="E24" s="59"/>
+      <c r="F24" s="13"/>
+      <c r="G24" s="15"/>
+      <c r="H24" s="37"/>
+      <c r="I24" s="60"/>
+      <c r="J24" s="61"/>
+      <c r="K24" s="47"/>
+      <c r="L24" s="38"/>
+      <c r="M24" s="16"/>
+      <c r="N24" s="49"/>
     </row>
     <row r="25" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="61" t="s">
+      <c r="A25" s="69" t="s">
         <v>33</v>
       </c>
-      <c r="B25" s="62"/>
-      <c r="C25" s="62"/>
-      <c r="D25" s="62"/>
-      <c r="E25" s="63"/>
-      <c r="F25" s="33"/>
-      <c r="G25" s="31">
+      <c r="B25" s="70"/>
+      <c r="C25" s="70"/>
+      <c r="D25" s="70"/>
+      <c r="E25" s="71"/>
+      <c r="F25" s="30"/>
+      <c r="G25" s="28">
         <f>SUM(G12:G24)</f>
         <v>0</v>
       </c>
-      <c r="H25" s="34"/>
-      <c r="I25" s="42" t="s">
+      <c r="H25" s="31"/>
+      <c r="I25" s="39" t="s">
         <v>32</v>
       </c>
-      <c r="J25" s="43"/>
-      <c r="K25" s="44">
+      <c r="J25" s="40"/>
+      <c r="K25" s="45">
         <f>SUM(K12:K24)</f>
         <v>0</v>
       </c>
-      <c r="L25" s="41"/>
-      <c r="M25" s="19"/>
-      <c r="N25" s="36"/>
+      <c r="L25" s="38"/>
+      <c r="M25" s="16"/>
+      <c r="N25" s="49"/>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A26" s="45" t="s">
+      <c r="A26" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="B26" s="59"/>
-      <c r="C26" s="59"/>
-      <c r="D26" s="59"/>
-      <c r="E26" s="46" t="s">
+      <c r="B26" s="62"/>
+      <c r="C26" s="62"/>
+      <c r="D26" s="62"/>
+      <c r="E26" s="42" t="s">
         <v>22</v>
       </c>
-      <c r="F26" s="47" t="s">
+      <c r="F26" s="43" t="s">
         <v>23</v>
       </c>
-      <c r="G26" s="89"/>
-      <c r="H26" s="89"/>
-      <c r="I26" s="89"/>
-      <c r="J26" s="89"/>
-      <c r="K26" s="48"/>
-      <c r="L26" s="48"/>
+      <c r="G26" s="66"/>
+      <c r="H26" s="66"/>
+      <c r="I26" s="66"/>
+      <c r="J26" s="66"/>
+      <c r="K26" s="44"/>
+      <c r="L26" s="44"/>
       <c r="M26" s="3"/>
       <c r="N26" s="5"/>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A27" s="20" t="s">
+      <c r="A27" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="B27" s="60"/>
-      <c r="C27" s="60"/>
-      <c r="D27" s="60"/>
-      <c r="E27" s="22"/>
-      <c r="F27" s="23"/>
-      <c r="G27" s="90"/>
-      <c r="H27" s="90"/>
-      <c r="I27" s="90"/>
-      <c r="J27" s="90"/>
-      <c r="K27" s="40"/>
-      <c r="L27" s="40"/>
-      <c r="M27" s="34"/>
-      <c r="N27" s="36"/>
+      <c r="B27" s="63"/>
+      <c r="C27" s="63"/>
+      <c r="D27" s="63"/>
+      <c r="E27" s="19"/>
+      <c r="F27" s="20"/>
+      <c r="G27" s="67"/>
+      <c r="H27" s="67"/>
+      <c r="I27" s="67"/>
+      <c r="J27" s="67"/>
+      <c r="K27" s="37"/>
+      <c r="L27" s="37"/>
+      <c r="M27" s="31"/>
+      <c r="N27" s="33"/>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A28" s="20" t="s">
+      <c r="A28" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="B28" s="94"/>
-      <c r="C28" s="94"/>
-      <c r="D28" s="94"/>
-      <c r="E28" s="95"/>
-      <c r="F28" s="23"/>
-      <c r="G28" s="90"/>
-      <c r="H28" s="90"/>
-      <c r="I28" s="90"/>
-      <c r="J28" s="90"/>
-      <c r="K28" s="40"/>
-      <c r="L28" s="37" t="s">
+      <c r="B28" s="64"/>
+      <c r="C28" s="64"/>
+      <c r="D28" s="64"/>
+      <c r="E28" s="65"/>
+      <c r="F28" s="20"/>
+      <c r="G28" s="67"/>
+      <c r="H28" s="67"/>
+      <c r="I28" s="67"/>
+      <c r="J28" s="67"/>
+      <c r="K28" s="37"/>
+      <c r="L28" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="M28" s="92"/>
-      <c r="N28" s="93"/>
+      <c r="M28" s="50"/>
+      <c r="N28" s="51"/>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A29" s="20" t="s">
+      <c r="A29" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="B29" s="51"/>
-      <c r="C29" s="51"/>
-      <c r="D29" s="51"/>
-      <c r="E29" s="22"/>
-      <c r="F29" s="23"/>
-      <c r="G29" s="90"/>
-      <c r="H29" s="90"/>
-      <c r="I29" s="90"/>
-      <c r="J29" s="90"/>
-      <c r="K29" s="40"/>
-      <c r="L29" s="37" t="s">
+      <c r="B29" s="52"/>
+      <c r="C29" s="52"/>
+      <c r="D29" s="52"/>
+      <c r="E29" s="19"/>
+      <c r="F29" s="20"/>
+      <c r="G29" s="67"/>
+      <c r="H29" s="67"/>
+      <c r="I29" s="67"/>
+      <c r="J29" s="67"/>
+      <c r="K29" s="37"/>
+      <c r="L29" s="34" t="s">
         <v>28</v>
       </c>
-      <c r="M29" s="49"/>
-      <c r="N29" s="50"/>
+      <c r="M29" s="53"/>
+      <c r="N29" s="54"/>
     </row>
     <row r="30" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="24" t="s">
+      <c r="A30" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="B30" s="52"/>
-      <c r="C30" s="52"/>
-      <c r="D30" s="52"/>
-      <c r="E30" s="26"/>
-      <c r="F30" s="27"/>
-      <c r="G30" s="91"/>
-      <c r="H30" s="91"/>
-      <c r="I30" s="91"/>
-      <c r="J30" s="91"/>
-      <c r="K30" s="28"/>
-      <c r="L30" s="29"/>
-      <c r="M30" s="25"/>
-      <c r="N30" s="30"/>
+      <c r="B30" s="55"/>
+      <c r="C30" s="55"/>
+      <c r="D30" s="55"/>
+      <c r="E30" s="23"/>
+      <c r="F30" s="24"/>
+      <c r="G30" s="68"/>
+      <c r="H30" s="68"/>
+      <c r="I30" s="68"/>
+      <c r="J30" s="68"/>
+      <c r="K30" s="25"/>
+      <c r="L30" s="26"/>
+      <c r="M30" s="22"/>
+      <c r="N30" s="27"/>
     </row>
   </sheetData>
   <mergeCells count="56">

</xml_diff>

<commit_message>
Extruder: Extruder Form Bulk Export modification and Fixed.
</commit_message>
<xml_diff>
--- a/app/views/extruder_form/records/extruder_report_format.xlsx
+++ b/app/views/extruder_form/records/extruder_report_format.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\MBPI-Projects\DEPLOYMENT-MixerExtruder-Project\app\views\extruder_form\records\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1B4EF37-9518-4D8D-86FA-FF21016B686C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13284681-1D65-4D6D-AD81-B38F20796051}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A8C50F24-49C3-4045-93FC-1EB156652CF7}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="34">
   <si>
     <t xml:space="preserve">MC# </t>
   </si>
@@ -224,7 +224,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="41">
+  <borders count="43">
     <border>
       <left/>
       <right/>
@@ -688,6 +688,32 @@
         <color indexed="64"/>
       </top>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -695,7 +721,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="97">
+  <cellXfs count="99">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -843,6 +869,9 @@
     </xf>
     <xf numFmtId="4" fontId="4" fillId="0" borderId="33" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="3" fillId="0" borderId="42" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -954,6 +983,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1287,13 +1319,13 @@
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
-      <c r="F5" s="76" t="s">
+      <c r="F5" s="77" t="s">
         <v>30</v>
       </c>
-      <c r="G5" s="77"/>
-      <c r="H5" s="77"/>
-      <c r="I5" s="77"/>
-      <c r="J5" s="78"/>
+      <c r="G5" s="78"/>
+      <c r="H5" s="78"/>
+      <c r="I5" s="78"/>
+      <c r="J5" s="79"/>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
@@ -1321,11 +1353,11 @@
       <c r="B7" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C7" s="79" t="s">
+      <c r="C7" s="80" t="s">
         <v>2</v>
       </c>
-      <c r="D7" s="80"/>
-      <c r="E7" s="81"/>
+      <c r="D7" s="81"/>
+      <c r="E7" s="82"/>
       <c r="F7" s="3" t="s">
         <v>3</v>
       </c>
@@ -1355,12 +1387,12 @@
       </c>
     </row>
     <row r="8" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="82"/>
-      <c r="B8" s="84"/>
-      <c r="C8" s="86"/>
-      <c r="D8" s="87"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="91"/>
+      <c r="A8" s="83"/>
+      <c r="B8" s="85"/>
+      <c r="C8" s="87"/>
+      <c r="D8" s="88"/>
+      <c r="E8" s="89"/>
+      <c r="F8" s="92"/>
       <c r="G8" s="31" t="s">
         <v>10</v>
       </c>
@@ -1387,12 +1419,12 @@
       </c>
     </row>
     <row r="9" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="83"/>
-      <c r="B9" s="85"/>
-      <c r="C9" s="89"/>
-      <c r="D9" s="90"/>
-      <c r="E9" s="85"/>
-      <c r="F9" s="89"/>
+      <c r="A9" s="84"/>
+      <c r="B9" s="86"/>
+      <c r="C9" s="90"/>
+      <c r="D9" s="91"/>
+      <c r="E9" s="86"/>
+      <c r="F9" s="90"/>
       <c r="G9" s="6"/>
       <c r="H9" s="6"/>
       <c r="I9" s="6"/>
@@ -1421,15 +1453,15 @@
       <c r="N10" s="33"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="92" t="s">
+      <c r="A11" s="93" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="72"/>
-      <c r="C11" s="73"/>
-      <c r="D11" s="93" t="s">
+      <c r="B11" s="73"/>
+      <c r="C11" s="74"/>
+      <c r="D11" s="94" t="s">
         <v>16</v>
       </c>
-      <c r="E11" s="59"/>
+      <c r="E11" s="60"/>
       <c r="F11" s="10" t="s">
         <v>17</v>
       </c>
@@ -1451,32 +1483,32 @@
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A12" s="94"/>
-      <c r="B12" s="72"/>
-      <c r="C12" s="73"/>
-      <c r="D12" s="58"/>
-      <c r="E12" s="59"/>
+      <c r="A12" s="95"/>
+      <c r="B12" s="73"/>
+      <c r="C12" s="74"/>
+      <c r="D12" s="59"/>
+      <c r="E12" s="60"/>
       <c r="F12" s="11"/>
       <c r="G12" s="12"/>
       <c r="H12" s="31"/>
-      <c r="I12" s="95"/>
-      <c r="J12" s="96"/>
+      <c r="I12" s="96"/>
+      <c r="J12" s="97"/>
       <c r="K12" s="46"/>
       <c r="L12" s="31"/>
       <c r="M12" s="13"/>
       <c r="N12" s="48"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A13" s="74"/>
-      <c r="B13" s="72"/>
-      <c r="C13" s="73"/>
-      <c r="D13" s="58"/>
-      <c r="E13" s="59"/>
+      <c r="A13" s="75"/>
+      <c r="B13" s="73"/>
+      <c r="C13" s="74"/>
+      <c r="D13" s="59"/>
+      <c r="E13" s="60"/>
       <c r="F13" s="14"/>
       <c r="G13" s="15"/>
       <c r="H13" s="35"/>
-      <c r="I13" s="60"/>
-      <c r="J13" s="61"/>
+      <c r="I13" s="61"/>
+      <c r="J13" s="62"/>
       <c r="K13" s="47"/>
       <c r="L13" s="31" t="s">
         <v>14</v>
@@ -1485,189 +1517,189 @@
       <c r="N13" s="49"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" s="74"/>
-      <c r="B14" s="72"/>
-      <c r="C14" s="73"/>
-      <c r="D14" s="58"/>
-      <c r="E14" s="59"/>
+      <c r="A14" s="75"/>
+      <c r="B14" s="73"/>
+      <c r="C14" s="74"/>
+      <c r="D14" s="59"/>
+      <c r="E14" s="60"/>
       <c r="F14" s="14"/>
       <c r="G14" s="15"/>
       <c r="H14" s="36"/>
-      <c r="I14" s="60"/>
-      <c r="J14" s="61"/>
+      <c r="I14" s="61"/>
+      <c r="J14" s="62"/>
       <c r="K14" s="47"/>
       <c r="L14" s="31"/>
       <c r="M14" s="16"/>
       <c r="N14" s="49"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" s="74"/>
-      <c r="B15" s="72"/>
-      <c r="C15" s="73"/>
-      <c r="D15" s="58"/>
-      <c r="E15" s="59"/>
+      <c r="A15" s="75"/>
+      <c r="B15" s="73"/>
+      <c r="C15" s="74"/>
+      <c r="D15" s="59"/>
+      <c r="E15" s="60"/>
       <c r="F15" s="14"/>
       <c r="G15" s="15"/>
       <c r="H15" s="36"/>
-      <c r="I15" s="60"/>
-      <c r="J15" s="61"/>
+      <c r="I15" s="61"/>
+      <c r="J15" s="62"/>
       <c r="K15" s="47"/>
       <c r="L15" s="31"/>
       <c r="M15" s="16"/>
       <c r="N15" s="49"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A16" s="74"/>
-      <c r="B16" s="72"/>
-      <c r="C16" s="73"/>
-      <c r="D16" s="75"/>
-      <c r="E16" s="59"/>
+      <c r="A16" s="75"/>
+      <c r="B16" s="73"/>
+      <c r="C16" s="74"/>
+      <c r="D16" s="76"/>
+      <c r="E16" s="60"/>
       <c r="F16" s="14"/>
       <c r="G16" s="15"/>
       <c r="H16" s="36"/>
-      <c r="I16" s="60"/>
-      <c r="J16" s="61"/>
+      <c r="I16" s="61"/>
+      <c r="J16" s="62"/>
       <c r="K16" s="47"/>
       <c r="L16" s="31"/>
       <c r="M16" s="16"/>
       <c r="N16" s="49"/>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A17" s="74"/>
-      <c r="B17" s="72"/>
-      <c r="C17" s="73"/>
-      <c r="D17" s="75"/>
-      <c r="E17" s="59"/>
+      <c r="A17" s="75"/>
+      <c r="B17" s="73"/>
+      <c r="C17" s="74"/>
+      <c r="D17" s="76"/>
+      <c r="E17" s="60"/>
       <c r="F17" s="14"/>
       <c r="G17" s="15"/>
       <c r="H17" s="36"/>
-      <c r="I17" s="60"/>
-      <c r="J17" s="61"/>
+      <c r="I17" s="61"/>
+      <c r="J17" s="62"/>
       <c r="K17" s="47"/>
       <c r="L17" s="31"/>
       <c r="M17" s="16"/>
       <c r="N17" s="49"/>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A18" s="74"/>
-      <c r="B18" s="72"/>
-      <c r="C18" s="73"/>
-      <c r="D18" s="58"/>
-      <c r="E18" s="59"/>
+      <c r="A18" s="75"/>
+      <c r="B18" s="73"/>
+      <c r="C18" s="74"/>
+      <c r="D18" s="59"/>
+      <c r="E18" s="60"/>
       <c r="F18" s="14"/>
       <c r="G18" s="15"/>
       <c r="H18" s="36"/>
-      <c r="I18" s="60"/>
-      <c r="J18" s="61"/>
+      <c r="I18" s="61"/>
+      <c r="J18" s="62"/>
       <c r="K18" s="47"/>
       <c r="L18" s="31"/>
       <c r="M18" s="16"/>
       <c r="N18" s="49"/>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A19" s="56"/>
-      <c r="B19" s="72"/>
-      <c r="C19" s="73"/>
-      <c r="D19" s="58"/>
-      <c r="E19" s="59"/>
+      <c r="A19" s="57"/>
+      <c r="B19" s="73"/>
+      <c r="C19" s="74"/>
+      <c r="D19" s="59"/>
+      <c r="E19" s="60"/>
       <c r="F19" s="14"/>
       <c r="G19" s="15"/>
       <c r="H19" s="37"/>
-      <c r="I19" s="60"/>
-      <c r="J19" s="61"/>
+      <c r="I19" s="61"/>
+      <c r="J19" s="62"/>
       <c r="K19" s="47"/>
       <c r="L19" s="38"/>
       <c r="M19" s="16"/>
       <c r="N19" s="49"/>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A20" s="56"/>
-      <c r="B20" s="72"/>
-      <c r="C20" s="73"/>
-      <c r="D20" s="58"/>
-      <c r="E20" s="59"/>
+      <c r="A20" s="57"/>
+      <c r="B20" s="73"/>
+      <c r="C20" s="74"/>
+      <c r="D20" s="59"/>
+      <c r="E20" s="60"/>
       <c r="F20" s="14"/>
       <c r="G20" s="15"/>
       <c r="H20" s="37"/>
-      <c r="I20" s="60"/>
-      <c r="J20" s="61"/>
+      <c r="I20" s="61"/>
+      <c r="J20" s="62"/>
       <c r="K20" s="47"/>
       <c r="L20" s="38"/>
       <c r="M20" s="16"/>
       <c r="N20" s="49"/>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A21" s="56"/>
-      <c r="B21" s="72"/>
-      <c r="C21" s="73"/>
-      <c r="D21" s="58"/>
-      <c r="E21" s="59"/>
+      <c r="A21" s="57"/>
+      <c r="B21" s="73"/>
+      <c r="C21" s="74"/>
+      <c r="D21" s="59"/>
+      <c r="E21" s="60"/>
       <c r="F21" s="14"/>
       <c r="G21" s="15"/>
       <c r="H21" s="37"/>
-      <c r="I21" s="60"/>
-      <c r="J21" s="61"/>
+      <c r="I21" s="61"/>
+      <c r="J21" s="62"/>
       <c r="K21" s="47"/>
       <c r="L21" s="38"/>
       <c r="M21" s="16"/>
       <c r="N21" s="49"/>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A22" s="56"/>
-      <c r="B22" s="72"/>
-      <c r="C22" s="73"/>
-      <c r="D22" s="58"/>
-      <c r="E22" s="59"/>
+      <c r="A22" s="57"/>
+      <c r="B22" s="73"/>
+      <c r="C22" s="74"/>
+      <c r="D22" s="59"/>
+      <c r="E22" s="60"/>
       <c r="F22" s="14"/>
       <c r="G22" s="15"/>
       <c r="H22" s="37"/>
-      <c r="I22" s="60"/>
-      <c r="J22" s="61"/>
+      <c r="I22" s="61"/>
+      <c r="J22" s="62"/>
       <c r="K22" s="47"/>
       <c r="L22" s="38"/>
       <c r="M22" s="16"/>
       <c r="N22" s="49"/>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A23" s="56"/>
-      <c r="B23" s="72"/>
-      <c r="C23" s="73"/>
-      <c r="D23" s="58"/>
-      <c r="E23" s="59"/>
+      <c r="A23" s="57"/>
+      <c r="B23" s="73"/>
+      <c r="C23" s="74"/>
+      <c r="D23" s="59"/>
+      <c r="E23" s="60"/>
       <c r="F23" s="14"/>
       <c r="G23" s="15"/>
       <c r="H23" s="37"/>
-      <c r="I23" s="60"/>
-      <c r="J23" s="61"/>
+      <c r="I23" s="61"/>
+      <c r="J23" s="62"/>
       <c r="K23" s="47"/>
       <c r="L23" s="38"/>
       <c r="M23" s="16"/>
       <c r="N23" s="49"/>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A24" s="56"/>
-      <c r="B24" s="57"/>
-      <c r="C24" s="57"/>
-      <c r="D24" s="58"/>
-      <c r="E24" s="59"/>
+      <c r="A24" s="57"/>
+      <c r="B24" s="58"/>
+      <c r="C24" s="58"/>
+      <c r="D24" s="59"/>
+      <c r="E24" s="60"/>
       <c r="F24" s="13"/>
       <c r="G24" s="15"/>
       <c r="H24" s="37"/>
-      <c r="I24" s="60"/>
-      <c r="J24" s="61"/>
+      <c r="I24" s="61"/>
+      <c r="J24" s="62"/>
       <c r="K24" s="47"/>
       <c r="L24" s="38"/>
       <c r="M24" s="16"/>
       <c r="N24" s="49"/>
     </row>
     <row r="25" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="69" t="s">
+      <c r="A25" s="70" t="s">
         <v>33</v>
       </c>
-      <c r="B25" s="70"/>
-      <c r="C25" s="70"/>
-      <c r="D25" s="70"/>
-      <c r="E25" s="71"/>
+      <c r="B25" s="71"/>
+      <c r="C25" s="71"/>
+      <c r="D25" s="71"/>
+      <c r="E25" s="72"/>
       <c r="F25" s="30"/>
       <c r="G25" s="28">
         <f>SUM(G12:G24)</f>
@@ -1683,26 +1715,31 @@
         <v>0</v>
       </c>
       <c r="L25" s="38"/>
-      <c r="M25" s="16"/>
-      <c r="N25" s="49"/>
+      <c r="M25" s="98" t="s">
+        <v>32</v>
+      </c>
+      <c r="N25" s="50">
+        <f>SUM(N12:N24)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="B26" s="62"/>
-      <c r="C26" s="62"/>
-      <c r="D26" s="62"/>
+      <c r="B26" s="63"/>
+      <c r="C26" s="63"/>
+      <c r="D26" s="63"/>
       <c r="E26" s="42" t="s">
         <v>22</v>
       </c>
       <c r="F26" s="43" t="s">
         <v>23</v>
       </c>
-      <c r="G26" s="66"/>
-      <c r="H26" s="66"/>
-      <c r="I26" s="66"/>
-      <c r="J26" s="66"/>
+      <c r="G26" s="67"/>
+      <c r="H26" s="67"/>
+      <c r="I26" s="67"/>
+      <c r="J26" s="67"/>
       <c r="K26" s="44"/>
       <c r="L26" s="44"/>
       <c r="M26" s="3"/>
@@ -1712,15 +1749,15 @@
       <c r="A27" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="B27" s="63"/>
-      <c r="C27" s="63"/>
-      <c r="D27" s="63"/>
+      <c r="B27" s="64"/>
+      <c r="C27" s="64"/>
+      <c r="D27" s="64"/>
       <c r="E27" s="19"/>
       <c r="F27" s="20"/>
-      <c r="G27" s="67"/>
-      <c r="H27" s="67"/>
-      <c r="I27" s="67"/>
-      <c r="J27" s="67"/>
+      <c r="G27" s="68"/>
+      <c r="H27" s="68"/>
+      <c r="I27" s="68"/>
+      <c r="J27" s="68"/>
       <c r="K27" s="37"/>
       <c r="L27" s="37"/>
       <c r="M27" s="31"/>
@@ -1730,55 +1767,55 @@
       <c r="A28" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="B28" s="64"/>
-      <c r="C28" s="64"/>
-      <c r="D28" s="64"/>
-      <c r="E28" s="65"/>
+      <c r="B28" s="65"/>
+      <c r="C28" s="65"/>
+      <c r="D28" s="65"/>
+      <c r="E28" s="66"/>
       <c r="F28" s="20"/>
-      <c r="G28" s="67"/>
-      <c r="H28" s="67"/>
-      <c r="I28" s="67"/>
-      <c r="J28" s="67"/>
+      <c r="G28" s="68"/>
+      <c r="H28" s="68"/>
+      <c r="I28" s="68"/>
+      <c r="J28" s="68"/>
       <c r="K28" s="37"/>
       <c r="L28" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="M28" s="50"/>
-      <c r="N28" s="51"/>
+      <c r="M28" s="51"/>
+      <c r="N28" s="52"/>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="B29" s="52"/>
-      <c r="C29" s="52"/>
-      <c r="D29" s="52"/>
+      <c r="B29" s="53"/>
+      <c r="C29" s="53"/>
+      <c r="D29" s="53"/>
       <c r="E29" s="19"/>
       <c r="F29" s="20"/>
-      <c r="G29" s="67"/>
-      <c r="H29" s="67"/>
-      <c r="I29" s="67"/>
-      <c r="J29" s="67"/>
+      <c r="G29" s="68"/>
+      <c r="H29" s="68"/>
+      <c r="I29" s="68"/>
+      <c r="J29" s="68"/>
       <c r="K29" s="37"/>
       <c r="L29" s="34" t="s">
         <v>28</v>
       </c>
-      <c r="M29" s="53"/>
-      <c r="N29" s="54"/>
+      <c r="M29" s="54"/>
+      <c r="N29" s="55"/>
     </row>
     <row r="30" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="B30" s="55"/>
-      <c r="C30" s="55"/>
-      <c r="D30" s="55"/>
+      <c r="B30" s="56"/>
+      <c r="C30" s="56"/>
+      <c r="D30" s="56"/>
       <c r="E30" s="23"/>
       <c r="F30" s="24"/>
-      <c r="G30" s="68"/>
-      <c r="H30" s="68"/>
-      <c r="I30" s="68"/>
-      <c r="J30" s="68"/>
+      <c r="G30" s="69"/>
+      <c r="H30" s="69"/>
+      <c r="I30" s="69"/>
+      <c r="J30" s="69"/>
       <c r="K30" s="25"/>
       <c r="L30" s="26"/>
       <c r="M30" s="22"/>

</xml_diff>

<commit_message>
Extruder Report: Bulk Export
</commit_message>
<xml_diff>
--- a/app/views/extruder_form/records/extruder_report_format.xlsx
+++ b/app/views/extruder_form/records/extruder_report_format.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\MBPI-Projects\DEPLOYMENT-MixerExtruder-Project\app\views\extruder_form\records\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13284681-1D65-4D6D-AD81-B38F20796051}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15502D2A-C464-421E-AD44-428F4DBF051D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A8C50F24-49C3-4045-93FC-1EB156652CF7}"/>
   </bookViews>
@@ -195,6 +195,7 @@
       <b/>
       <sz val="8"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -224,7 +225,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="43">
+  <borders count="45">
     <border>
       <left/>
       <right/>
@@ -712,6 +713,26 @@
         <color indexed="64"/>
       </top>
       <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="8"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -721,7 +742,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="99">
+  <cellXfs count="101">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -873,6 +894,9 @@
     <xf numFmtId="4" fontId="3" fillId="0" borderId="42" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -897,44 +921,50 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="43" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="44" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="35" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="3" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="3" fillId="0" borderId="31" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
     <xf numFmtId="167" fontId="4" fillId="0" borderId="30" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="35" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="16" fontId="3" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="3" fillId="0" borderId="31" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="168" fontId="4" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -983,9 +1013,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1319,13 +1346,13 @@
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
-      <c r="F5" s="77" t="s">
+      <c r="F5" s="80" t="s">
         <v>30</v>
       </c>
-      <c r="G5" s="78"/>
-      <c r="H5" s="78"/>
-      <c r="I5" s="78"/>
-      <c r="J5" s="79"/>
+      <c r="G5" s="81"/>
+      <c r="H5" s="81"/>
+      <c r="I5" s="81"/>
+      <c r="J5" s="82"/>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
@@ -1353,11 +1380,11 @@
       <c r="B7" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C7" s="80" t="s">
+      <c r="C7" s="83" t="s">
         <v>2</v>
       </c>
-      <c r="D7" s="81"/>
-      <c r="E7" s="82"/>
+      <c r="D7" s="84"/>
+      <c r="E7" s="85"/>
       <c r="F7" s="3" t="s">
         <v>3</v>
       </c>
@@ -1387,12 +1414,12 @@
       </c>
     </row>
     <row r="8" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="83"/>
-      <c r="B8" s="85"/>
-      <c r="C8" s="87"/>
-      <c r="D8" s="88"/>
-      <c r="E8" s="89"/>
-      <c r="F8" s="92"/>
+      <c r="A8" s="86"/>
+      <c r="B8" s="88"/>
+      <c r="C8" s="90"/>
+      <c r="D8" s="91"/>
+      <c r="E8" s="92"/>
+      <c r="F8" s="95"/>
       <c r="G8" s="31" t="s">
         <v>10</v>
       </c>
@@ -1419,12 +1446,12 @@
       </c>
     </row>
     <row r="9" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="84"/>
-      <c r="B9" s="86"/>
-      <c r="C9" s="90"/>
-      <c r="D9" s="91"/>
-      <c r="E9" s="86"/>
-      <c r="F9" s="90"/>
+      <c r="A9" s="87"/>
+      <c r="B9" s="89"/>
+      <c r="C9" s="93"/>
+      <c r="D9" s="94"/>
+      <c r="E9" s="89"/>
+      <c r="F9" s="93"/>
       <c r="G9" s="6"/>
       <c r="H9" s="6"/>
       <c r="I9" s="6"/>
@@ -1453,15 +1480,15 @@
       <c r="N10" s="33"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="93" t="s">
+      <c r="A11" s="96" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="73"/>
-      <c r="C11" s="74"/>
-      <c r="D11" s="94" t="s">
+      <c r="B11" s="74"/>
+      <c r="C11" s="75"/>
+      <c r="D11" s="97" t="s">
         <v>16</v>
       </c>
-      <c r="E11" s="60"/>
+      <c r="E11" s="61"/>
       <c r="F11" s="10" t="s">
         <v>17</v>
       </c>
@@ -1483,32 +1510,32 @@
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A12" s="95"/>
-      <c r="B12" s="73"/>
-      <c r="C12" s="74"/>
-      <c r="D12" s="59"/>
-      <c r="E12" s="60"/>
+      <c r="A12" s="98"/>
+      <c r="B12" s="74"/>
+      <c r="C12" s="75"/>
+      <c r="D12" s="60"/>
+      <c r="E12" s="61"/>
       <c r="F12" s="11"/>
       <c r="G12" s="12"/>
       <c r="H12" s="31"/>
-      <c r="I12" s="96"/>
-      <c r="J12" s="97"/>
+      <c r="I12" s="99"/>
+      <c r="J12" s="100"/>
       <c r="K12" s="46"/>
       <c r="L12" s="31"/>
       <c r="M12" s="13"/>
       <c r="N12" s="48"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A13" s="75"/>
-      <c r="B13" s="73"/>
-      <c r="C13" s="74"/>
-      <c r="D13" s="59"/>
-      <c r="E13" s="60"/>
+      <c r="A13" s="78"/>
+      <c r="B13" s="74"/>
+      <c r="C13" s="75"/>
+      <c r="D13" s="60"/>
+      <c r="E13" s="61"/>
       <c r="F13" s="14"/>
       <c r="G13" s="15"/>
       <c r="H13" s="35"/>
-      <c r="I13" s="61"/>
-      <c r="J13" s="62"/>
+      <c r="I13" s="76"/>
+      <c r="J13" s="77"/>
       <c r="K13" s="47"/>
       <c r="L13" s="31" t="s">
         <v>14</v>
@@ -1517,189 +1544,189 @@
       <c r="N13" s="49"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" s="75"/>
-      <c r="B14" s="73"/>
-      <c r="C14" s="74"/>
-      <c r="D14" s="59"/>
-      <c r="E14" s="60"/>
+      <c r="A14" s="78"/>
+      <c r="B14" s="74"/>
+      <c r="C14" s="75"/>
+      <c r="D14" s="60"/>
+      <c r="E14" s="61"/>
       <c r="F14" s="14"/>
       <c r="G14" s="15"/>
       <c r="H14" s="36"/>
-      <c r="I14" s="61"/>
-      <c r="J14" s="62"/>
+      <c r="I14" s="76"/>
+      <c r="J14" s="77"/>
       <c r="K14" s="47"/>
       <c r="L14" s="31"/>
       <c r="M14" s="16"/>
       <c r="N14" s="49"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" s="75"/>
-      <c r="B15" s="73"/>
-      <c r="C15" s="74"/>
-      <c r="D15" s="59"/>
-      <c r="E15" s="60"/>
+      <c r="A15" s="78"/>
+      <c r="B15" s="74"/>
+      <c r="C15" s="75"/>
+      <c r="D15" s="60"/>
+      <c r="E15" s="61"/>
       <c r="F15" s="14"/>
       <c r="G15" s="15"/>
       <c r="H15" s="36"/>
-      <c r="I15" s="61"/>
-      <c r="J15" s="62"/>
+      <c r="I15" s="76"/>
+      <c r="J15" s="77"/>
       <c r="K15" s="47"/>
       <c r="L15" s="31"/>
       <c r="M15" s="16"/>
       <c r="N15" s="49"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A16" s="75"/>
-      <c r="B16" s="73"/>
-      <c r="C16" s="74"/>
-      <c r="D16" s="76"/>
-      <c r="E16" s="60"/>
+      <c r="A16" s="78"/>
+      <c r="B16" s="74"/>
+      <c r="C16" s="75"/>
+      <c r="D16" s="79"/>
+      <c r="E16" s="61"/>
       <c r="F16" s="14"/>
       <c r="G16" s="15"/>
       <c r="H16" s="36"/>
-      <c r="I16" s="61"/>
-      <c r="J16" s="62"/>
+      <c r="I16" s="76"/>
+      <c r="J16" s="77"/>
       <c r="K16" s="47"/>
       <c r="L16" s="31"/>
       <c r="M16" s="16"/>
       <c r="N16" s="49"/>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A17" s="75"/>
-      <c r="B17" s="73"/>
-      <c r="C17" s="74"/>
-      <c r="D17" s="76"/>
-      <c r="E17" s="60"/>
+      <c r="A17" s="78"/>
+      <c r="B17" s="74"/>
+      <c r="C17" s="75"/>
+      <c r="D17" s="79"/>
+      <c r="E17" s="61"/>
       <c r="F17" s="14"/>
       <c r="G17" s="15"/>
       <c r="H17" s="36"/>
-      <c r="I17" s="61"/>
-      <c r="J17" s="62"/>
+      <c r="I17" s="76"/>
+      <c r="J17" s="77"/>
       <c r="K17" s="47"/>
       <c r="L17" s="31"/>
       <c r="M17" s="16"/>
       <c r="N17" s="49"/>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A18" s="75"/>
-      <c r="B18" s="73"/>
-      <c r="C18" s="74"/>
-      <c r="D18" s="59"/>
-      <c r="E18" s="60"/>
+      <c r="A18" s="78"/>
+      <c r="B18" s="74"/>
+      <c r="C18" s="75"/>
+      <c r="D18" s="60"/>
+      <c r="E18" s="61"/>
       <c r="F18" s="14"/>
       <c r="G18" s="15"/>
       <c r="H18" s="36"/>
-      <c r="I18" s="61"/>
-      <c r="J18" s="62"/>
+      <c r="I18" s="76"/>
+      <c r="J18" s="77"/>
       <c r="K18" s="47"/>
       <c r="L18" s="31"/>
       <c r="M18" s="16"/>
       <c r="N18" s="49"/>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A19" s="57"/>
-      <c r="B19" s="73"/>
-      <c r="C19" s="74"/>
-      <c r="D19" s="59"/>
-      <c r="E19" s="60"/>
+      <c r="A19" s="58"/>
+      <c r="B19" s="74"/>
+      <c r="C19" s="75"/>
+      <c r="D19" s="60"/>
+      <c r="E19" s="61"/>
       <c r="F19" s="14"/>
       <c r="G19" s="15"/>
       <c r="H19" s="37"/>
-      <c r="I19" s="61"/>
-      <c r="J19" s="62"/>
+      <c r="I19" s="76"/>
+      <c r="J19" s="77"/>
       <c r="K19" s="47"/>
       <c r="L19" s="38"/>
       <c r="M19" s="16"/>
       <c r="N19" s="49"/>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A20" s="57"/>
-      <c r="B20" s="73"/>
-      <c r="C20" s="74"/>
-      <c r="D20" s="59"/>
-      <c r="E20" s="60"/>
+      <c r="A20" s="58"/>
+      <c r="B20" s="74"/>
+      <c r="C20" s="75"/>
+      <c r="D20" s="60"/>
+      <c r="E20" s="61"/>
       <c r="F20" s="14"/>
       <c r="G20" s="15"/>
       <c r="H20" s="37"/>
-      <c r="I20" s="61"/>
-      <c r="J20" s="62"/>
+      <c r="I20" s="76"/>
+      <c r="J20" s="77"/>
       <c r="K20" s="47"/>
       <c r="L20" s="38"/>
       <c r="M20" s="16"/>
       <c r="N20" s="49"/>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A21" s="57"/>
-      <c r="B21" s="73"/>
-      <c r="C21" s="74"/>
-      <c r="D21" s="59"/>
-      <c r="E21" s="60"/>
+      <c r="A21" s="58"/>
+      <c r="B21" s="74"/>
+      <c r="C21" s="75"/>
+      <c r="D21" s="60"/>
+      <c r="E21" s="61"/>
       <c r="F21" s="14"/>
       <c r="G21" s="15"/>
       <c r="H21" s="37"/>
-      <c r="I21" s="61"/>
-      <c r="J21" s="62"/>
+      <c r="I21" s="76"/>
+      <c r="J21" s="77"/>
       <c r="K21" s="47"/>
       <c r="L21" s="38"/>
       <c r="M21" s="16"/>
       <c r="N21" s="49"/>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A22" s="57"/>
-      <c r="B22" s="73"/>
-      <c r="C22" s="74"/>
-      <c r="D22" s="59"/>
-      <c r="E22" s="60"/>
+      <c r="A22" s="58"/>
+      <c r="B22" s="74"/>
+      <c r="C22" s="75"/>
+      <c r="D22" s="60"/>
+      <c r="E22" s="61"/>
       <c r="F22" s="14"/>
       <c r="G22" s="15"/>
       <c r="H22" s="37"/>
-      <c r="I22" s="61"/>
-      <c r="J22" s="62"/>
+      <c r="I22" s="76"/>
+      <c r="J22" s="77"/>
       <c r="K22" s="47"/>
       <c r="L22" s="38"/>
       <c r="M22" s="16"/>
       <c r="N22" s="49"/>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A23" s="57"/>
-      <c r="B23" s="73"/>
-      <c r="C23" s="74"/>
-      <c r="D23" s="59"/>
-      <c r="E23" s="60"/>
+      <c r="A23" s="58"/>
+      <c r="B23" s="74"/>
+      <c r="C23" s="75"/>
+      <c r="D23" s="60"/>
+      <c r="E23" s="61"/>
       <c r="F23" s="14"/>
       <c r="G23" s="15"/>
       <c r="H23" s="37"/>
-      <c r="I23" s="61"/>
-      <c r="J23" s="62"/>
+      <c r="I23" s="76"/>
+      <c r="J23" s="77"/>
       <c r="K23" s="47"/>
       <c r="L23" s="38"/>
       <c r="M23" s="16"/>
       <c r="N23" s="49"/>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A24" s="57"/>
-      <c r="B24" s="58"/>
-      <c r="C24" s="58"/>
-      <c r="D24" s="59"/>
-      <c r="E24" s="60"/>
+      <c r="A24" s="58"/>
+      <c r="B24" s="59"/>
+      <c r="C24" s="59"/>
+      <c r="D24" s="60"/>
+      <c r="E24" s="61"/>
       <c r="F24" s="13"/>
       <c r="G24" s="15"/>
       <c r="H24" s="37"/>
-      <c r="I24" s="61"/>
-      <c r="J24" s="62"/>
+      <c r="I24" s="62"/>
+      <c r="J24" s="63"/>
       <c r="K24" s="47"/>
       <c r="L24" s="38"/>
       <c r="M24" s="16"/>
       <c r="N24" s="49"/>
     </row>
     <row r="25" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="70" t="s">
+      <c r="A25" s="71" t="s">
         <v>33</v>
       </c>
-      <c r="B25" s="71"/>
-      <c r="C25" s="71"/>
-      <c r="D25" s="71"/>
-      <c r="E25" s="72"/>
+      <c r="B25" s="72"/>
+      <c r="C25" s="72"/>
+      <c r="D25" s="72"/>
+      <c r="E25" s="73"/>
       <c r="F25" s="30"/>
       <c r="G25" s="28">
         <f>SUM(G12:G24)</f>
@@ -1715,7 +1742,7 @@
         <v>0</v>
       </c>
       <c r="L25" s="38"/>
-      <c r="M25" s="98" t="s">
+      <c r="M25" s="51" t="s">
         <v>32</v>
       </c>
       <c r="N25" s="50">
@@ -1727,19 +1754,19 @@
       <c r="A26" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="B26" s="63"/>
-      <c r="C26" s="63"/>
-      <c r="D26" s="63"/>
+      <c r="B26" s="64"/>
+      <c r="C26" s="64"/>
+      <c r="D26" s="64"/>
       <c r="E26" s="42" t="s">
         <v>22</v>
       </c>
       <c r="F26" s="43" t="s">
         <v>23</v>
       </c>
-      <c r="G26" s="67"/>
-      <c r="H26" s="67"/>
-      <c r="I26" s="67"/>
-      <c r="J26" s="67"/>
+      <c r="G26" s="68"/>
+      <c r="H26" s="68"/>
+      <c r="I26" s="68"/>
+      <c r="J26" s="68"/>
       <c r="K26" s="44"/>
       <c r="L26" s="44"/>
       <c r="M26" s="3"/>
@@ -1749,15 +1776,15 @@
       <c r="A27" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="B27" s="64"/>
-      <c r="C27" s="64"/>
-      <c r="D27" s="64"/>
+      <c r="B27" s="65"/>
+      <c r="C27" s="65"/>
+      <c r="D27" s="65"/>
       <c r="E27" s="19"/>
       <c r="F27" s="20"/>
-      <c r="G27" s="68"/>
-      <c r="H27" s="68"/>
-      <c r="I27" s="68"/>
-      <c r="J27" s="68"/>
+      <c r="G27" s="69"/>
+      <c r="H27" s="69"/>
+      <c r="I27" s="69"/>
+      <c r="J27" s="69"/>
       <c r="K27" s="37"/>
       <c r="L27" s="37"/>
       <c r="M27" s="31"/>
@@ -1767,55 +1794,55 @@
       <c r="A28" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="B28" s="65"/>
-      <c r="C28" s="65"/>
-      <c r="D28" s="65"/>
-      <c r="E28" s="66"/>
+      <c r="B28" s="66"/>
+      <c r="C28" s="66"/>
+      <c r="D28" s="66"/>
+      <c r="E28" s="67"/>
       <c r="F28" s="20"/>
-      <c r="G28" s="68"/>
-      <c r="H28" s="68"/>
-      <c r="I28" s="68"/>
-      <c r="J28" s="68"/>
+      <c r="G28" s="69"/>
+      <c r="H28" s="69"/>
+      <c r="I28" s="69"/>
+      <c r="J28" s="69"/>
       <c r="K28" s="37"/>
       <c r="L28" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="M28" s="51"/>
-      <c r="N28" s="52"/>
+      <c r="M28" s="52"/>
+      <c r="N28" s="53"/>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="B29" s="53"/>
-      <c r="C29" s="53"/>
-      <c r="D29" s="53"/>
+      <c r="B29" s="54"/>
+      <c r="C29" s="54"/>
+      <c r="D29" s="54"/>
       <c r="E29" s="19"/>
       <c r="F29" s="20"/>
-      <c r="G29" s="68"/>
-      <c r="H29" s="68"/>
-      <c r="I29" s="68"/>
-      <c r="J29" s="68"/>
+      <c r="G29" s="69"/>
+      <c r="H29" s="69"/>
+      <c r="I29" s="69"/>
+      <c r="J29" s="69"/>
       <c r="K29" s="37"/>
       <c r="L29" s="34" t="s">
         <v>28</v>
       </c>
-      <c r="M29" s="54"/>
-      <c r="N29" s="55"/>
+      <c r="M29" s="55"/>
+      <c r="N29" s="56"/>
     </row>
     <row r="30" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="B30" s="56"/>
-      <c r="C30" s="56"/>
-      <c r="D30" s="56"/>
+      <c r="B30" s="57"/>
+      <c r="C30" s="57"/>
+      <c r="D30" s="57"/>
       <c r="E30" s="23"/>
       <c r="F30" s="24"/>
-      <c r="G30" s="69"/>
-      <c r="H30" s="69"/>
-      <c r="I30" s="69"/>
-      <c r="J30" s="69"/>
+      <c r="G30" s="70"/>
+      <c r="H30" s="70"/>
+      <c r="I30" s="70"/>
+      <c r="J30" s="70"/>
       <c r="K30" s="25"/>
       <c r="L30" s="26"/>
       <c r="M30" s="22"/>

</xml_diff>

<commit_message>
Extruder Report: Completed fixing the bug in the Extruder Report
</commit_message>
<xml_diff>
--- a/app/views/extruder_form/records/extruder_report_format.xlsx
+++ b/app/views/extruder_form/records/extruder_report_format.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\MBPI-Projects\DEPLOYMENT-MixerExtruder-Project\app\views\extruder_form\records\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15502D2A-C464-421E-AD44-428F4DBF051D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E899706-52CB-429D-9EA7-EDACACEA29F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A8C50F24-49C3-4045-93FC-1EB156652CF7}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="35">
   <si>
     <t xml:space="preserve">MC# </t>
   </si>
@@ -111,9 +111,6 @@
     <t>Time :</t>
   </si>
   <si>
-    <t>Resins :</t>
-  </si>
-  <si>
     <t>Operator:</t>
   </si>
   <si>
@@ -123,9 +120,6 @@
     <t>Supervisor:</t>
   </si>
   <si>
-    <t>Palletizer:</t>
-  </si>
-  <si>
     <t xml:space="preserve">Extruder Machine No. </t>
   </si>
   <si>
@@ -136,6 +130,15 @@
   </si>
   <si>
     <t xml:space="preserve">Total   </t>
+  </si>
+  <si>
+    <t>Pelletizer:</t>
+  </si>
+  <si>
+    <t>Resins Purged:</t>
+  </si>
+  <si>
+    <t>Resin used (carrier):</t>
   </si>
 </sst>
 </file>
@@ -225,7 +228,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="45">
+  <borders count="46">
     <border>
       <left/>
       <right/>
@@ -421,21 +424,6 @@
       <top/>
       <bottom style="thin">
         <color indexed="8"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -647,21 +635,6 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
       <right/>
       <top style="thin">
         <color indexed="64"/>
@@ -732,6 +705,41 @@
       <left/>
       <right/>
       <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="8"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -742,7 +750,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="101">
+  <cellXfs count="109">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -771,160 +779,153 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="4" fillId="0" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="4" fillId="0" borderId="32" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="35" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="169" fontId="4" fillId="0" borderId="33" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="34" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="34" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="3" fillId="0" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="3" fillId="3" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="21" fontId="3" fillId="0" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="38" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="34" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="35" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="35" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="3" fillId="0" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="3" fillId="3" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="21" fontId="3" fillId="0" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="38" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="3" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="3" fillId="0" borderId="37" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="4" fillId="0" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="40" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="40" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="3" fillId="0" borderId="39" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="4" fillId="0" borderId="26" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="4" fillId="0" borderId="31" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="4" fillId="0" borderId="28" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="4" fillId="0" borderId="33" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="3" fillId="0" borderId="42" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="30" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="27" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="32" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="3" fillId="0" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="41" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="4" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="43" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="44" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="42" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -936,7 +937,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -945,30 +946,16 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="35" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="34" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="16" fontId="3" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="3" fillId="0" borderId="31" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="30" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="29" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="167" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="31" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -984,7 +971,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -999,20 +985,74 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="3" fillId="0" borderId="33" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="3" fillId="0" borderId="34" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="3" fillId="0" borderId="44" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="4" fillId="0" borderId="45" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="4" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="4" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="45" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="45" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="45" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1329,12 +1369,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12E9B9F7-E023-41F8-9561-3EC2FB8099F6}">
-  <dimension ref="A4:N30"/>
+  <dimension ref="A4:N31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="2.28515625" customWidth="1"/>
     <col min="5" max="5" width="14.140625" customWidth="1"/>
     <col min="10" max="10" width="12.85546875" customWidth="1"/>
+    <col min="12" max="12" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="18.42578125" customWidth="1"/>
     <col min="14" max="14" width="13.28515625" customWidth="1"/>
   </cols>
@@ -1346,13 +1388,13 @@
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
-      <c r="F5" s="80" t="s">
-        <v>30</v>
-      </c>
-      <c r="G5" s="81"/>
-      <c r="H5" s="81"/>
-      <c r="I5" s="81"/>
-      <c r="J5" s="82"/>
+      <c r="F5" s="71" t="s">
+        <v>28</v>
+      </c>
+      <c r="G5" s="72"/>
+      <c r="H5" s="72"/>
+      <c r="I5" s="72"/>
+      <c r="J5" s="73"/>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
@@ -1380,16 +1422,16 @@
       <c r="B7" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C7" s="83" t="s">
+      <c r="C7" s="74" t="s">
         <v>2</v>
       </c>
-      <c r="D7" s="84"/>
-      <c r="E7" s="85"/>
+      <c r="D7" s="75"/>
+      <c r="E7" s="76"/>
       <c r="F7" s="3" t="s">
         <v>3</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="H7" s="3" t="s">
         <v>5</v>
@@ -1414,12 +1456,12 @@
       </c>
     </row>
     <row r="8" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="86"/>
-      <c r="B8" s="88"/>
-      <c r="C8" s="90"/>
-      <c r="D8" s="91"/>
-      <c r="E8" s="92"/>
-      <c r="F8" s="95"/>
+      <c r="A8" s="108"/>
+      <c r="B8" s="78"/>
+      <c r="C8" s="80"/>
+      <c r="D8" s="81"/>
+      <c r="E8" s="82"/>
+      <c r="F8" s="85"/>
       <c r="G8" s="31" t="s">
         <v>10</v>
       </c>
@@ -1442,16 +1484,16 @@
         <v>10</v>
       </c>
       <c r="N8" s="18" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="87"/>
-      <c r="B9" s="89"/>
-      <c r="C9" s="93"/>
-      <c r="D9" s="94"/>
-      <c r="E9" s="89"/>
-      <c r="F9" s="93"/>
+      <c r="A9" s="77"/>
+      <c r="B9" s="79"/>
+      <c r="C9" s="83"/>
+      <c r="D9" s="84"/>
+      <c r="E9" s="79"/>
+      <c r="F9" s="83"/>
       <c r="G9" s="6"/>
       <c r="H9" s="6"/>
       <c r="I9" s="6"/>
@@ -1480,15 +1522,15 @@
       <c r="N10" s="33"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="96" t="s">
+      <c r="A11" s="105" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="74"/>
-      <c r="C11" s="75"/>
-      <c r="D11" s="97" t="s">
+      <c r="B11" s="106"/>
+      <c r="C11" s="107"/>
+      <c r="D11" s="86" t="s">
         <v>16</v>
       </c>
-      <c r="E11" s="61"/>
+      <c r="E11" s="58"/>
       <c r="F11" s="10" t="s">
         <v>17</v>
       </c>
@@ -1510,32 +1552,32 @@
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A12" s="98"/>
-      <c r="B12" s="74"/>
-      <c r="C12" s="75"/>
-      <c r="D12" s="60"/>
-      <c r="E12" s="61"/>
+      <c r="A12" s="102"/>
+      <c r="B12" s="103"/>
+      <c r="C12" s="104"/>
+      <c r="D12" s="57"/>
+      <c r="E12" s="58"/>
       <c r="F12" s="11"/>
       <c r="G12" s="12"/>
       <c r="H12" s="31"/>
-      <c r="I12" s="99"/>
-      <c r="J12" s="100"/>
+      <c r="I12" s="87"/>
+      <c r="J12" s="88"/>
       <c r="K12" s="46"/>
       <c r="L12" s="31"/>
       <c r="M12" s="13"/>
       <c r="N12" s="48"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A13" s="78"/>
-      <c r="B13" s="74"/>
-      <c r="C13" s="75"/>
-      <c r="D13" s="60"/>
-      <c r="E13" s="61"/>
+      <c r="A13" s="99"/>
+      <c r="B13" s="100"/>
+      <c r="C13" s="101"/>
+      <c r="D13" s="57"/>
+      <c r="E13" s="58"/>
       <c r="F13" s="14"/>
       <c r="G13" s="15"/>
       <c r="H13" s="35"/>
-      <c r="I13" s="76"/>
-      <c r="J13" s="77"/>
+      <c r="I13" s="68"/>
+      <c r="J13" s="69"/>
       <c r="K13" s="47"/>
       <c r="L13" s="31" t="s">
         <v>14</v>
@@ -1544,189 +1586,189 @@
       <c r="N13" s="49"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" s="78"/>
-      <c r="B14" s="74"/>
-      <c r="C14" s="75"/>
-      <c r="D14" s="60"/>
-      <c r="E14" s="61"/>
+      <c r="A14" s="99"/>
+      <c r="B14" s="100"/>
+      <c r="C14" s="101"/>
+      <c r="D14" s="57"/>
+      <c r="E14" s="58"/>
       <c r="F14" s="14"/>
       <c r="G14" s="15"/>
       <c r="H14" s="36"/>
-      <c r="I14" s="76"/>
-      <c r="J14" s="77"/>
+      <c r="I14" s="68"/>
+      <c r="J14" s="69"/>
       <c r="K14" s="47"/>
       <c r="L14" s="31"/>
       <c r="M14" s="16"/>
       <c r="N14" s="49"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" s="78"/>
-      <c r="B15" s="74"/>
-      <c r="C15" s="75"/>
-      <c r="D15" s="60"/>
-      <c r="E15" s="61"/>
+      <c r="A15" s="99"/>
+      <c r="B15" s="100"/>
+      <c r="C15" s="101"/>
+      <c r="D15" s="57"/>
+      <c r="E15" s="58"/>
       <c r="F15" s="14"/>
       <c r="G15" s="15"/>
       <c r="H15" s="36"/>
-      <c r="I15" s="76"/>
-      <c r="J15" s="77"/>
+      <c r="I15" s="68"/>
+      <c r="J15" s="69"/>
       <c r="K15" s="47"/>
       <c r="L15" s="31"/>
       <c r="M15" s="16"/>
       <c r="N15" s="49"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A16" s="78"/>
-      <c r="B16" s="74"/>
-      <c r="C16" s="75"/>
-      <c r="D16" s="79"/>
-      <c r="E16" s="61"/>
+      <c r="A16" s="99"/>
+      <c r="B16" s="100"/>
+      <c r="C16" s="101"/>
+      <c r="D16" s="70"/>
+      <c r="E16" s="58"/>
       <c r="F16" s="14"/>
       <c r="G16" s="15"/>
       <c r="H16" s="36"/>
-      <c r="I16" s="76"/>
-      <c r="J16" s="77"/>
+      <c r="I16" s="68"/>
+      <c r="J16" s="69"/>
       <c r="K16" s="47"/>
       <c r="L16" s="31"/>
       <c r="M16" s="16"/>
       <c r="N16" s="49"/>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A17" s="78"/>
-      <c r="B17" s="74"/>
-      <c r="C17" s="75"/>
-      <c r="D17" s="79"/>
-      <c r="E17" s="61"/>
+      <c r="A17" s="99"/>
+      <c r="B17" s="100"/>
+      <c r="C17" s="101"/>
+      <c r="D17" s="70"/>
+      <c r="E17" s="58"/>
       <c r="F17" s="14"/>
       <c r="G17" s="15"/>
       <c r="H17" s="36"/>
-      <c r="I17" s="76"/>
-      <c r="J17" s="77"/>
+      <c r="I17" s="68"/>
+      <c r="J17" s="69"/>
       <c r="K17" s="47"/>
       <c r="L17" s="31"/>
       <c r="M17" s="16"/>
       <c r="N17" s="49"/>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A18" s="78"/>
-      <c r="B18" s="74"/>
-      <c r="C18" s="75"/>
-      <c r="D18" s="60"/>
-      <c r="E18" s="61"/>
+      <c r="A18" s="99"/>
+      <c r="B18" s="100"/>
+      <c r="C18" s="101"/>
+      <c r="D18" s="57"/>
+      <c r="E18" s="58"/>
       <c r="F18" s="14"/>
       <c r="G18" s="15"/>
       <c r="H18" s="36"/>
-      <c r="I18" s="76"/>
-      <c r="J18" s="77"/>
+      <c r="I18" s="68"/>
+      <c r="J18" s="69"/>
       <c r="K18" s="47"/>
       <c r="L18" s="31"/>
       <c r="M18" s="16"/>
       <c r="N18" s="49"/>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A19" s="58"/>
-      <c r="B19" s="74"/>
-      <c r="C19" s="75"/>
-      <c r="D19" s="60"/>
-      <c r="E19" s="61"/>
+      <c r="A19" s="96"/>
+      <c r="B19" s="97"/>
+      <c r="C19" s="98"/>
+      <c r="D19" s="57"/>
+      <c r="E19" s="58"/>
       <c r="F19" s="14"/>
       <c r="G19" s="15"/>
       <c r="H19" s="37"/>
-      <c r="I19" s="76"/>
-      <c r="J19" s="77"/>
+      <c r="I19" s="68"/>
+      <c r="J19" s="69"/>
       <c r="K19" s="47"/>
       <c r="L19" s="38"/>
       <c r="M19" s="16"/>
       <c r="N19" s="49"/>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A20" s="58"/>
-      <c r="B20" s="74"/>
-      <c r="C20" s="75"/>
-      <c r="D20" s="60"/>
-      <c r="E20" s="61"/>
+      <c r="A20" s="96"/>
+      <c r="B20" s="97"/>
+      <c r="C20" s="98"/>
+      <c r="D20" s="57"/>
+      <c r="E20" s="58"/>
       <c r="F20" s="14"/>
       <c r="G20" s="15"/>
       <c r="H20" s="37"/>
-      <c r="I20" s="76"/>
-      <c r="J20" s="77"/>
+      <c r="I20" s="68"/>
+      <c r="J20" s="69"/>
       <c r="K20" s="47"/>
       <c r="L20" s="38"/>
       <c r="M20" s="16"/>
       <c r="N20" s="49"/>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A21" s="58"/>
-      <c r="B21" s="74"/>
-      <c r="C21" s="75"/>
-      <c r="D21" s="60"/>
-      <c r="E21" s="61"/>
+      <c r="A21" s="96"/>
+      <c r="B21" s="97"/>
+      <c r="C21" s="98"/>
+      <c r="D21" s="57"/>
+      <c r="E21" s="58"/>
       <c r="F21" s="14"/>
       <c r="G21" s="15"/>
       <c r="H21" s="37"/>
-      <c r="I21" s="76"/>
-      <c r="J21" s="77"/>
+      <c r="I21" s="68"/>
+      <c r="J21" s="69"/>
       <c r="K21" s="47"/>
       <c r="L21" s="38"/>
       <c r="M21" s="16"/>
       <c r="N21" s="49"/>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A22" s="58"/>
-      <c r="B22" s="74"/>
-      <c r="C22" s="75"/>
-      <c r="D22" s="60"/>
-      <c r="E22" s="61"/>
+      <c r="A22" s="96"/>
+      <c r="B22" s="97"/>
+      <c r="C22" s="98"/>
+      <c r="D22" s="57"/>
+      <c r="E22" s="58"/>
       <c r="F22" s="14"/>
       <c r="G22" s="15"/>
       <c r="H22" s="37"/>
-      <c r="I22" s="76"/>
-      <c r="J22" s="77"/>
+      <c r="I22" s="68"/>
+      <c r="J22" s="69"/>
       <c r="K22" s="47"/>
       <c r="L22" s="38"/>
       <c r="M22" s="16"/>
       <c r="N22" s="49"/>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A23" s="58"/>
-      <c r="B23" s="74"/>
-      <c r="C23" s="75"/>
-      <c r="D23" s="60"/>
-      <c r="E23" s="61"/>
+      <c r="A23" s="96"/>
+      <c r="B23" s="97"/>
+      <c r="C23" s="98"/>
+      <c r="D23" s="57"/>
+      <c r="E23" s="58"/>
       <c r="F23" s="14"/>
       <c r="G23" s="15"/>
       <c r="H23" s="37"/>
-      <c r="I23" s="76"/>
-      <c r="J23" s="77"/>
+      <c r="I23" s="68"/>
+      <c r="J23" s="69"/>
       <c r="K23" s="47"/>
       <c r="L23" s="38"/>
       <c r="M23" s="16"/>
       <c r="N23" s="49"/>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A24" s="58"/>
-      <c r="B24" s="59"/>
-      <c r="C24" s="59"/>
-      <c r="D24" s="60"/>
-      <c r="E24" s="61"/>
+      <c r="A24" s="96"/>
+      <c r="B24" s="97"/>
+      <c r="C24" s="98"/>
+      <c r="D24" s="57"/>
+      <c r="E24" s="58"/>
       <c r="F24" s="13"/>
       <c r="G24" s="15"/>
       <c r="H24" s="37"/>
-      <c r="I24" s="62"/>
-      <c r="J24" s="63"/>
+      <c r="I24" s="59"/>
+      <c r="J24" s="60"/>
       <c r="K24" s="47"/>
       <c r="L24" s="38"/>
       <c r="M24" s="16"/>
       <c r="N24" s="49"/>
     </row>
     <row r="25" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="71" t="s">
-        <v>33</v>
-      </c>
-      <c r="B25" s="72"/>
-      <c r="C25" s="72"/>
-      <c r="D25" s="72"/>
-      <c r="E25" s="73"/>
+      <c r="A25" s="93" t="s">
+        <v>31</v>
+      </c>
+      <c r="B25" s="94"/>
+      <c r="C25" s="94"/>
+      <c r="D25" s="94"/>
+      <c r="E25" s="95"/>
       <c r="F25" s="30"/>
       <c r="G25" s="28">
         <f>SUM(G12:G24)</f>
@@ -1734,7 +1776,7 @@
       </c>
       <c r="H25" s="31"/>
       <c r="I25" s="39" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="J25" s="40"/>
       <c r="K25" s="45">
@@ -1743,7 +1785,7 @@
       </c>
       <c r="L25" s="38"/>
       <c r="M25" s="51" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="N25" s="50">
         <f>SUM(N12:N24)</f>
@@ -1754,19 +1796,19 @@
       <c r="A26" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="B26" s="64"/>
-      <c r="C26" s="64"/>
-      <c r="D26" s="64"/>
+      <c r="B26" s="61"/>
+      <c r="C26" s="61"/>
+      <c r="D26" s="61"/>
       <c r="E26" s="42" t="s">
         <v>22</v>
       </c>
       <c r="F26" s="43" t="s">
         <v>23</v>
       </c>
-      <c r="G26" s="68"/>
-      <c r="H26" s="68"/>
-      <c r="I26" s="68"/>
-      <c r="J26" s="68"/>
+      <c r="G26" s="65"/>
+      <c r="H26" s="65"/>
+      <c r="I26" s="65"/>
+      <c r="J26" s="65"/>
       <c r="K26" s="44"/>
       <c r="L26" s="44"/>
       <c r="M26" s="3"/>
@@ -1776,15 +1818,15 @@
       <c r="A27" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="B27" s="65"/>
-      <c r="C27" s="65"/>
-      <c r="D27" s="65"/>
+      <c r="B27" s="62"/>
+      <c r="C27" s="62"/>
+      <c r="D27" s="62"/>
       <c r="E27" s="19"/>
       <c r="F27" s="20"/>
-      <c r="G27" s="69"/>
-      <c r="H27" s="69"/>
-      <c r="I27" s="69"/>
-      <c r="J27" s="69"/>
+      <c r="G27" s="66"/>
+      <c r="H27" s="66"/>
+      <c r="I27" s="66"/>
+      <c r="J27" s="66"/>
       <c r="K27" s="37"/>
       <c r="L27" s="37"/>
       <c r="M27" s="31"/>
@@ -1792,64 +1834,82 @@
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="B28" s="63"/>
+      <c r="C28" s="63"/>
+      <c r="D28" s="63"/>
+      <c r="E28" s="64"/>
+      <c r="F28" s="20"/>
+      <c r="G28" s="66"/>
+      <c r="H28" s="66"/>
+      <c r="I28" s="66"/>
+      <c r="J28" s="66"/>
+      <c r="K28" s="37"/>
+      <c r="L28" s="91" t="s">
         <v>25</v>
       </c>
-      <c r="B28" s="66"/>
-      <c r="C28" s="66"/>
-      <c r="D28" s="66"/>
-      <c r="E28" s="67"/>
-      <c r="F28" s="20"/>
-      <c r="G28" s="69"/>
-      <c r="H28" s="69"/>
-      <c r="I28" s="69"/>
-      <c r="J28" s="69"/>
-      <c r="K28" s="37"/>
-      <c r="L28" s="34" t="s">
+      <c r="M28" s="92"/>
+      <c r="N28" s="64"/>
+    </row>
+    <row r="29" spans="1:14" ht="23.25" x14ac:dyDescent="0.25">
+      <c r="A29" s="90" t="s">
+        <v>34</v>
+      </c>
+      <c r="B29" s="89"/>
+      <c r="C29" s="89"/>
+      <c r="D29" s="89"/>
+      <c r="E29" s="52"/>
+      <c r="F29" s="20"/>
+      <c r="G29" s="66"/>
+      <c r="H29" s="66"/>
+      <c r="I29" s="66"/>
+      <c r="J29" s="66"/>
+      <c r="K29" s="37"/>
+      <c r="L29" s="91"/>
+      <c r="M29" s="92"/>
+      <c r="N29" s="64"/>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A30" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="M28" s="52"/>
-      <c r="N28" s="53"/>
-    </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A29" s="17" t="s">
+      <c r="B30" s="53"/>
+      <c r="C30" s="53"/>
+      <c r="D30" s="53"/>
+      <c r="E30" s="19"/>
+      <c r="F30" s="20"/>
+      <c r="G30" s="66"/>
+      <c r="H30" s="66"/>
+      <c r="I30" s="66"/>
+      <c r="J30" s="66"/>
+      <c r="K30" s="37"/>
+      <c r="L30" s="34" t="s">
         <v>27</v>
       </c>
-      <c r="B29" s="54"/>
-      <c r="C29" s="54"/>
-      <c r="D29" s="54"/>
-      <c r="E29" s="19"/>
-      <c r="F29" s="20"/>
-      <c r="G29" s="69"/>
-      <c r="H29" s="69"/>
-      <c r="I29" s="69"/>
-      <c r="J29" s="69"/>
-      <c r="K29" s="37"/>
-      <c r="L29" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="M29" s="55"/>
-      <c r="N29" s="56"/>
-    </row>
-    <row r="30" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="21" t="s">
-        <v>29</v>
-      </c>
-      <c r="B30" s="57"/>
-      <c r="C30" s="57"/>
-      <c r="D30" s="57"/>
-      <c r="E30" s="23"/>
-      <c r="F30" s="24"/>
-      <c r="G30" s="70"/>
-      <c r="H30" s="70"/>
-      <c r="I30" s="70"/>
-      <c r="J30" s="70"/>
-      <c r="K30" s="25"/>
-      <c r="L30" s="26"/>
-      <c r="M30" s="22"/>
-      <c r="N30" s="27"/>
+      <c r="M30" s="54"/>
+      <c r="N30" s="55"/>
+    </row>
+    <row r="31" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="21" t="s">
+        <v>32</v>
+      </c>
+      <c r="B31" s="56"/>
+      <c r="C31" s="56"/>
+      <c r="D31" s="56"/>
+      <c r="E31" s="23"/>
+      <c r="F31" s="24"/>
+      <c r="G31" s="67"/>
+      <c r="H31" s="67"/>
+      <c r="I31" s="67"/>
+      <c r="J31" s="67"/>
+      <c r="K31" s="25"/>
+      <c r="L31" s="26"/>
+      <c r="M31" s="22"/>
+      <c r="N31" s="27"/>
     </row>
   </sheetData>
-  <mergeCells count="56">
+  <mergeCells count="58">
     <mergeCell ref="A13:C13"/>
     <mergeCell ref="D13:E13"/>
     <mergeCell ref="I13:J13"/>
@@ -1894,18 +1954,20 @@
     <mergeCell ref="A23:C23"/>
     <mergeCell ref="D23:E23"/>
     <mergeCell ref="I23:J23"/>
-    <mergeCell ref="M28:N28"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="M29:N29"/>
     <mergeCell ref="B30:D30"/>
+    <mergeCell ref="M30:N30"/>
+    <mergeCell ref="B31:D31"/>
     <mergeCell ref="A24:C24"/>
     <mergeCell ref="D24:E24"/>
     <mergeCell ref="I24:J24"/>
     <mergeCell ref="B26:D26"/>
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="B28:E28"/>
-    <mergeCell ref="G26:J30"/>
+    <mergeCell ref="G26:J31"/>
     <mergeCell ref="A25:E25"/>
+    <mergeCell ref="M28:N29"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="L28:L29"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="5" scale="110" fitToWidth="0" orientation="landscape" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
Extruder Records Bulk Export: Completed and Debugged the Feature
</commit_message>
<xml_diff>
--- a/app/views/extruder_form/records/extruder_report_format.xlsx
+++ b/app/views/extruder_form/records/extruder_report_format.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\MBPI-Projects\DEPLOYMENT-MixerExtruder-Project\app\views\extruder_form\records\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E899706-52CB-429D-9EA7-EDACACEA29F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67CCD491-C946-4469-B068-67A86ED77FD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A8C50F24-49C3-4045-93FC-1EB156652CF7}"/>
   </bookViews>
@@ -632,17 +632,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right style="thin">
         <color indexed="8"/>
@@ -741,6 +730,17 @@
         <color indexed="64"/>
       </top>
       <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -866,25 +866,19 @@
     <xf numFmtId="4" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="4" fillId="0" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="38" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="37" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="38" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="37" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="168" fontId="3" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="4" fontId="3" fillId="0" borderId="37" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="3" fillId="0" borderId="36" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="4" fillId="0" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -897,66 +891,41 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="4" fontId="4" fillId="0" borderId="32" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="3" fillId="0" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="3" fillId="0" borderId="39" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="44" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="41" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="42" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="34" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="167" fontId="4" fillId="0" borderId="29" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="167" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="31" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -968,6 +937,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -985,7 +957,25 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="44" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="44" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="167" fontId="4" fillId="0" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -994,65 +984,75 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="31" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="4" fillId="0" borderId="44" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="4" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="4" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="41" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="34" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="3" fillId="0" borderId="33" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="3" fillId="0" borderId="34" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="3" fillId="0" borderId="43" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="16" fontId="3" fillId="0" borderId="33" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="3" fillId="0" borderId="34" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="3" fillId="0" borderId="44" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="4" fillId="0" borderId="45" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="4" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="4" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="45" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="45" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="45" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1376,6 +1376,7 @@
     <col min="3" max="3" width="2.28515625" customWidth="1"/>
     <col min="5" max="5" width="14.140625" customWidth="1"/>
     <col min="10" max="10" width="12.85546875" customWidth="1"/>
+    <col min="11" max="11" width="13" customWidth="1"/>
     <col min="12" max="12" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="18.42578125" customWidth="1"/>
     <col min="14" max="14" width="13.28515625" customWidth="1"/>
@@ -1388,13 +1389,13 @@
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
-      <c r="F5" s="71" t="s">
+      <c r="F5" s="60" t="s">
         <v>28</v>
       </c>
-      <c r="G5" s="72"/>
-      <c r="H5" s="72"/>
-      <c r="I5" s="72"/>
-      <c r="J5" s="73"/>
+      <c r="G5" s="61"/>
+      <c r="H5" s="61"/>
+      <c r="I5" s="61"/>
+      <c r="J5" s="62"/>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
@@ -1422,11 +1423,11 @@
       <c r="B7" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C7" s="74" t="s">
+      <c r="C7" s="63" t="s">
         <v>2</v>
       </c>
-      <c r="D7" s="75"/>
-      <c r="E7" s="76"/>
+      <c r="D7" s="64"/>
+      <c r="E7" s="65"/>
       <c r="F7" s="3" t="s">
         <v>3</v>
       </c>
@@ -1456,12 +1457,12 @@
       </c>
     </row>
     <row r="8" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="108"/>
-      <c r="B8" s="78"/>
-      <c r="C8" s="80"/>
-      <c r="D8" s="81"/>
-      <c r="E8" s="82"/>
-      <c r="F8" s="85"/>
+      <c r="A8" s="66"/>
+      <c r="B8" s="68"/>
+      <c r="C8" s="70"/>
+      <c r="D8" s="71"/>
+      <c r="E8" s="72"/>
+      <c r="F8" s="75"/>
       <c r="G8" s="31" t="s">
         <v>10</v>
       </c>
@@ -1488,12 +1489,12 @@
       </c>
     </row>
     <row r="9" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="77"/>
-      <c r="B9" s="79"/>
-      <c r="C9" s="83"/>
-      <c r="D9" s="84"/>
-      <c r="E9" s="79"/>
-      <c r="F9" s="83"/>
+      <c r="A9" s="67"/>
+      <c r="B9" s="69"/>
+      <c r="C9" s="73"/>
+      <c r="D9" s="74"/>
+      <c r="E9" s="69"/>
+      <c r="F9" s="73"/>
       <c r="G9" s="6"/>
       <c r="H9" s="6"/>
       <c r="I9" s="6"/>
@@ -1522,15 +1523,15 @@
       <c r="N10" s="33"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="105" t="s">
+      <c r="A11" s="76" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="106"/>
-      <c r="C11" s="107"/>
-      <c r="D11" s="86" t="s">
+      <c r="B11" s="77"/>
+      <c r="C11" s="78"/>
+      <c r="D11" s="79" t="s">
         <v>16</v>
       </c>
-      <c r="E11" s="58"/>
+      <c r="E11" s="57"/>
       <c r="F11" s="10" t="s">
         <v>17</v>
       </c>
@@ -1552,265 +1553,265 @@
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A12" s="102"/>
-      <c r="B12" s="103"/>
-      <c r="C12" s="104"/>
-      <c r="D12" s="57"/>
-      <c r="E12" s="58"/>
+      <c r="A12" s="80"/>
+      <c r="B12" s="81"/>
+      <c r="C12" s="82"/>
+      <c r="D12" s="56"/>
+      <c r="E12" s="57"/>
       <c r="F12" s="11"/>
       <c r="G12" s="12"/>
       <c r="H12" s="31"/>
-      <c r="I12" s="87"/>
-      <c r="J12" s="88"/>
-      <c r="K12" s="46"/>
+      <c r="I12" s="83"/>
+      <c r="J12" s="84"/>
+      <c r="K12" s="44"/>
       <c r="L12" s="31"/>
       <c r="M12" s="13"/>
-      <c r="N12" s="48"/>
+      <c r="N12" s="46"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A13" s="99"/>
-      <c r="B13" s="100"/>
-      <c r="C13" s="101"/>
-      <c r="D13" s="57"/>
-      <c r="E13" s="58"/>
+      <c r="A13" s="53"/>
+      <c r="B13" s="54"/>
+      <c r="C13" s="55"/>
+      <c r="D13" s="56"/>
+      <c r="E13" s="57"/>
       <c r="F13" s="14"/>
       <c r="G13" s="15"/>
       <c r="H13" s="35"/>
-      <c r="I13" s="68"/>
-      <c r="J13" s="69"/>
-      <c r="K13" s="47"/>
+      <c r="I13" s="58"/>
+      <c r="J13" s="59"/>
+      <c r="K13" s="45"/>
       <c r="L13" s="31" t="s">
         <v>14</v>
       </c>
       <c r="M13" s="16"/>
-      <c r="N13" s="49"/>
+      <c r="N13" s="47"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" s="99"/>
-      <c r="B14" s="100"/>
-      <c r="C14" s="101"/>
-      <c r="D14" s="57"/>
-      <c r="E14" s="58"/>
+      <c r="A14" s="53"/>
+      <c r="B14" s="54"/>
+      <c r="C14" s="55"/>
+      <c r="D14" s="56"/>
+      <c r="E14" s="57"/>
       <c r="F14" s="14"/>
       <c r="G14" s="15"/>
       <c r="H14" s="36"/>
-      <c r="I14" s="68"/>
-      <c r="J14" s="69"/>
-      <c r="K14" s="47"/>
+      <c r="I14" s="58"/>
+      <c r="J14" s="59"/>
+      <c r="K14" s="45"/>
       <c r="L14" s="31"/>
       <c r="M14" s="16"/>
-      <c r="N14" s="49"/>
+      <c r="N14" s="47"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" s="99"/>
-      <c r="B15" s="100"/>
-      <c r="C15" s="101"/>
-      <c r="D15" s="57"/>
-      <c r="E15" s="58"/>
+      <c r="A15" s="53"/>
+      <c r="B15" s="54"/>
+      <c r="C15" s="55"/>
+      <c r="D15" s="56"/>
+      <c r="E15" s="57"/>
       <c r="F15" s="14"/>
       <c r="G15" s="15"/>
       <c r="H15" s="36"/>
-      <c r="I15" s="68"/>
-      <c r="J15" s="69"/>
-      <c r="K15" s="47"/>
+      <c r="I15" s="58"/>
+      <c r="J15" s="59"/>
+      <c r="K15" s="45"/>
       <c r="L15" s="31"/>
       <c r="M15" s="16"/>
-      <c r="N15" s="49"/>
+      <c r="N15" s="47"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A16" s="99"/>
-      <c r="B16" s="100"/>
-      <c r="C16" s="101"/>
-      <c r="D16" s="70"/>
-      <c r="E16" s="58"/>
+      <c r="A16" s="53"/>
+      <c r="B16" s="54"/>
+      <c r="C16" s="55"/>
+      <c r="D16" s="85"/>
+      <c r="E16" s="57"/>
       <c r="F16" s="14"/>
       <c r="G16" s="15"/>
       <c r="H16" s="36"/>
-      <c r="I16" s="68"/>
-      <c r="J16" s="69"/>
-      <c r="K16" s="47"/>
+      <c r="I16" s="58"/>
+      <c r="J16" s="59"/>
+      <c r="K16" s="45"/>
       <c r="L16" s="31"/>
       <c r="M16" s="16"/>
-      <c r="N16" s="49"/>
+      <c r="N16" s="47"/>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A17" s="99"/>
-      <c r="B17" s="100"/>
-      <c r="C17" s="101"/>
-      <c r="D17" s="70"/>
-      <c r="E17" s="58"/>
+      <c r="A17" s="53"/>
+      <c r="B17" s="54"/>
+      <c r="C17" s="55"/>
+      <c r="D17" s="85"/>
+      <c r="E17" s="57"/>
       <c r="F17" s="14"/>
       <c r="G17" s="15"/>
       <c r="H17" s="36"/>
-      <c r="I17" s="68"/>
-      <c r="J17" s="69"/>
-      <c r="K17" s="47"/>
+      <c r="I17" s="58"/>
+      <c r="J17" s="59"/>
+      <c r="K17" s="45"/>
       <c r="L17" s="31"/>
       <c r="M17" s="16"/>
-      <c r="N17" s="49"/>
+      <c r="N17" s="47"/>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A18" s="99"/>
-      <c r="B18" s="100"/>
-      <c r="C18" s="101"/>
-      <c r="D18" s="57"/>
-      <c r="E18" s="58"/>
+      <c r="A18" s="53"/>
+      <c r="B18" s="54"/>
+      <c r="C18" s="55"/>
+      <c r="D18" s="56"/>
+      <c r="E18" s="57"/>
       <c r="F18" s="14"/>
       <c r="G18" s="15"/>
       <c r="H18" s="36"/>
-      <c r="I18" s="68"/>
-      <c r="J18" s="69"/>
-      <c r="K18" s="47"/>
+      <c r="I18" s="58"/>
+      <c r="J18" s="59"/>
+      <c r="K18" s="45"/>
       <c r="L18" s="31"/>
       <c r="M18" s="16"/>
-      <c r="N18" s="49"/>
+      <c r="N18" s="47"/>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A19" s="96"/>
-      <c r="B19" s="97"/>
-      <c r="C19" s="98"/>
-      <c r="D19" s="57"/>
-      <c r="E19" s="58"/>
+      <c r="A19" s="86"/>
+      <c r="B19" s="87"/>
+      <c r="C19" s="88"/>
+      <c r="D19" s="56"/>
+      <c r="E19" s="57"/>
       <c r="F19" s="14"/>
       <c r="G19" s="15"/>
       <c r="H19" s="37"/>
-      <c r="I19" s="68"/>
-      <c r="J19" s="69"/>
-      <c r="K19" s="47"/>
+      <c r="I19" s="58"/>
+      <c r="J19" s="59"/>
+      <c r="K19" s="45"/>
       <c r="L19" s="38"/>
       <c r="M19" s="16"/>
-      <c r="N19" s="49"/>
+      <c r="N19" s="47"/>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A20" s="96"/>
-      <c r="B20" s="97"/>
-      <c r="C20" s="98"/>
-      <c r="D20" s="57"/>
-      <c r="E20" s="58"/>
+      <c r="A20" s="86"/>
+      <c r="B20" s="87"/>
+      <c r="C20" s="88"/>
+      <c r="D20" s="56"/>
+      <c r="E20" s="57"/>
       <c r="F20" s="14"/>
       <c r="G20" s="15"/>
       <c r="H20" s="37"/>
-      <c r="I20" s="68"/>
-      <c r="J20" s="69"/>
-      <c r="K20" s="47"/>
+      <c r="I20" s="58"/>
+      <c r="J20" s="59"/>
+      <c r="K20" s="45"/>
       <c r="L20" s="38"/>
       <c r="M20" s="16"/>
-      <c r="N20" s="49"/>
+      <c r="N20" s="47"/>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A21" s="96"/>
-      <c r="B21" s="97"/>
-      <c r="C21" s="98"/>
-      <c r="D21" s="57"/>
-      <c r="E21" s="58"/>
+      <c r="A21" s="86"/>
+      <c r="B21" s="87"/>
+      <c r="C21" s="88"/>
+      <c r="D21" s="56"/>
+      <c r="E21" s="57"/>
       <c r="F21" s="14"/>
       <c r="G21" s="15"/>
       <c r="H21" s="37"/>
-      <c r="I21" s="68"/>
-      <c r="J21" s="69"/>
-      <c r="K21" s="47"/>
+      <c r="I21" s="58"/>
+      <c r="J21" s="59"/>
+      <c r="K21" s="45"/>
       <c r="L21" s="38"/>
       <c r="M21" s="16"/>
-      <c r="N21" s="49"/>
+      <c r="N21" s="47"/>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A22" s="96"/>
-      <c r="B22" s="97"/>
-      <c r="C22" s="98"/>
-      <c r="D22" s="57"/>
-      <c r="E22" s="58"/>
+      <c r="A22" s="86"/>
+      <c r="B22" s="87"/>
+      <c r="C22" s="88"/>
+      <c r="D22" s="56"/>
+      <c r="E22" s="57"/>
       <c r="F22" s="14"/>
       <c r="G22" s="15"/>
       <c r="H22" s="37"/>
-      <c r="I22" s="68"/>
-      <c r="J22" s="69"/>
-      <c r="K22" s="47"/>
+      <c r="I22" s="58"/>
+      <c r="J22" s="59"/>
+      <c r="K22" s="45"/>
       <c r="L22" s="38"/>
       <c r="M22" s="16"/>
-      <c r="N22" s="49"/>
+      <c r="N22" s="47"/>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A23" s="96"/>
-      <c r="B23" s="97"/>
-      <c r="C23" s="98"/>
-      <c r="D23" s="57"/>
-      <c r="E23" s="58"/>
+      <c r="A23" s="86"/>
+      <c r="B23" s="87"/>
+      <c r="C23" s="88"/>
+      <c r="D23" s="56"/>
+      <c r="E23" s="57"/>
       <c r="F23" s="14"/>
       <c r="G23" s="15"/>
       <c r="H23" s="37"/>
-      <c r="I23" s="68"/>
-      <c r="J23" s="69"/>
-      <c r="K23" s="47"/>
+      <c r="I23" s="58"/>
+      <c r="J23" s="59"/>
+      <c r="K23" s="45"/>
       <c r="L23" s="38"/>
       <c r="M23" s="16"/>
-      <c r="N23" s="49"/>
+      <c r="N23" s="47"/>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A24" s="96"/>
-      <c r="B24" s="97"/>
-      <c r="C24" s="98"/>
-      <c r="D24" s="57"/>
-      <c r="E24" s="58"/>
+      <c r="A24" s="86"/>
+      <c r="B24" s="87"/>
+      <c r="C24" s="88"/>
+      <c r="D24" s="56"/>
+      <c r="E24" s="57"/>
       <c r="F24" s="13"/>
       <c r="G24" s="15"/>
       <c r="H24" s="37"/>
-      <c r="I24" s="59"/>
-      <c r="J24" s="60"/>
-      <c r="K24" s="47"/>
+      <c r="I24" s="93"/>
+      <c r="J24" s="94"/>
+      <c r="K24" s="45"/>
       <c r="L24" s="38"/>
       <c r="M24" s="16"/>
-      <c r="N24" s="49"/>
+      <c r="N24" s="47"/>
     </row>
     <row r="25" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="93" t="s">
+      <c r="A25" s="102" t="s">
         <v>31</v>
       </c>
-      <c r="B25" s="94"/>
-      <c r="C25" s="94"/>
-      <c r="D25" s="94"/>
-      <c r="E25" s="95"/>
+      <c r="B25" s="103"/>
+      <c r="C25" s="103"/>
+      <c r="D25" s="103"/>
+      <c r="E25" s="104"/>
       <c r="F25" s="30"/>
       <c r="G25" s="28">
         <f>SUM(G12:G24)</f>
         <v>0</v>
       </c>
       <c r="H25" s="31"/>
-      <c r="I25" s="39" t="s">
+      <c r="I25" s="107" t="s">
         <v>30</v>
       </c>
-      <c r="J25" s="40"/>
-      <c r="K25" s="45">
+      <c r="J25" s="108"/>
+      <c r="K25" s="43">
         <f>SUM(K12:K24)</f>
         <v>0</v>
       </c>
-      <c r="L25" s="38"/>
-      <c r="M25" s="51" t="s">
+      <c r="L25" s="51"/>
+      <c r="M25" s="50" t="s">
         <v>30</v>
       </c>
-      <c r="N25" s="50">
+      <c r="N25" s="52">
         <f>SUM(N12:N24)</f>
         <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A26" s="41" t="s">
+      <c r="A26" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="B26" s="61"/>
-      <c r="C26" s="61"/>
-      <c r="D26" s="61"/>
-      <c r="E26" s="42" t="s">
+      <c r="B26" s="95"/>
+      <c r="C26" s="95"/>
+      <c r="D26" s="95"/>
+      <c r="E26" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="F26" s="43" t="s">
+      <c r="F26" s="41" t="s">
         <v>23</v>
       </c>
-      <c r="G26" s="65"/>
-      <c r="H26" s="65"/>
-      <c r="I26" s="65"/>
-      <c r="J26" s="65"/>
-      <c r="K26" s="44"/>
-      <c r="L26" s="44"/>
+      <c r="G26" s="99"/>
+      <c r="H26" s="99"/>
+      <c r="I26" s="99"/>
+      <c r="J26" s="99"/>
+      <c r="K26" s="42"/>
+      <c r="L26" s="42"/>
       <c r="M26" s="3"/>
       <c r="N26" s="5"/>
     </row>
@@ -1818,15 +1819,15 @@
       <c r="A27" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="B27" s="62"/>
-      <c r="C27" s="62"/>
-      <c r="D27" s="62"/>
+      <c r="B27" s="96"/>
+      <c r="C27" s="96"/>
+      <c r="D27" s="96"/>
       <c r="E27" s="19"/>
       <c r="F27" s="20"/>
-      <c r="G27" s="66"/>
-      <c r="H27" s="66"/>
-      <c r="I27" s="66"/>
-      <c r="J27" s="66"/>
+      <c r="G27" s="100"/>
+      <c r="H27" s="100"/>
+      <c r="I27" s="100"/>
+      <c r="J27" s="100"/>
       <c r="K27" s="37"/>
       <c r="L27" s="37"/>
       <c r="M27" s="31"/>
@@ -1836,73 +1837,73 @@
       <c r="A28" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="B28" s="63"/>
-      <c r="C28" s="63"/>
-      <c r="D28" s="63"/>
-      <c r="E28" s="64"/>
+      <c r="B28" s="97"/>
+      <c r="C28" s="97"/>
+      <c r="D28" s="97"/>
+      <c r="E28" s="98"/>
       <c r="F28" s="20"/>
-      <c r="G28" s="66"/>
-      <c r="H28" s="66"/>
-      <c r="I28" s="66"/>
-      <c r="J28" s="66"/>
+      <c r="G28" s="100"/>
+      <c r="H28" s="100"/>
+      <c r="I28" s="100"/>
+      <c r="J28" s="100"/>
       <c r="K28" s="37"/>
-      <c r="L28" s="91" t="s">
+      <c r="L28" s="106" t="s">
         <v>25</v>
       </c>
-      <c r="M28" s="92"/>
-      <c r="N28" s="64"/>
+      <c r="M28" s="97"/>
+      <c r="N28" s="98"/>
     </row>
     <row r="29" spans="1:14" ht="23.25" x14ac:dyDescent="0.25">
-      <c r="A29" s="90" t="s">
+      <c r="A29" s="49" t="s">
         <v>34</v>
       </c>
-      <c r="B29" s="89"/>
-      <c r="C29" s="89"/>
-      <c r="D29" s="89"/>
-      <c r="E29" s="52"/>
+      <c r="B29" s="105"/>
+      <c r="C29" s="105"/>
+      <c r="D29" s="105"/>
+      <c r="E29" s="48"/>
       <c r="F29" s="20"/>
-      <c r="G29" s="66"/>
-      <c r="H29" s="66"/>
-      <c r="I29" s="66"/>
-      <c r="J29" s="66"/>
+      <c r="G29" s="100"/>
+      <c r="H29" s="100"/>
+      <c r="I29" s="100"/>
+      <c r="J29" s="100"/>
       <c r="K29" s="37"/>
-      <c r="L29" s="91"/>
-      <c r="M29" s="92"/>
-      <c r="N29" s="64"/>
+      <c r="L29" s="106"/>
+      <c r="M29" s="97"/>
+      <c r="N29" s="98"/>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="B30" s="53"/>
-      <c r="C30" s="53"/>
-      <c r="D30" s="53"/>
+      <c r="B30" s="89"/>
+      <c r="C30" s="89"/>
+      <c r="D30" s="89"/>
       <c r="E30" s="19"/>
       <c r="F30" s="20"/>
-      <c r="G30" s="66"/>
-      <c r="H30" s="66"/>
-      <c r="I30" s="66"/>
-      <c r="J30" s="66"/>
+      <c r="G30" s="100"/>
+      <c r="H30" s="100"/>
+      <c r="I30" s="100"/>
+      <c r="J30" s="100"/>
       <c r="K30" s="37"/>
       <c r="L30" s="34" t="s">
         <v>27</v>
       </c>
-      <c r="M30" s="54"/>
-      <c r="N30" s="55"/>
+      <c r="M30" s="90"/>
+      <c r="N30" s="91"/>
     </row>
     <row r="31" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="B31" s="56"/>
-      <c r="C31" s="56"/>
-      <c r="D31" s="56"/>
+      <c r="B31" s="92"/>
+      <c r="C31" s="92"/>
+      <c r="D31" s="92"/>
       <c r="E31" s="23"/>
       <c r="F31" s="24"/>
-      <c r="G31" s="67"/>
-      <c r="H31" s="67"/>
-      <c r="I31" s="67"/>
-      <c r="J31" s="67"/>
+      <c r="G31" s="101"/>
+      <c r="H31" s="101"/>
+      <c r="I31" s="101"/>
+      <c r="J31" s="101"/>
       <c r="K31" s="25"/>
       <c r="L31" s="26"/>
       <c r="M31" s="22"/>
@@ -1910,6 +1911,50 @@
     </row>
   </sheetData>
   <mergeCells count="58">
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="M30:N30"/>
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="I24:J24"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="B28:E28"/>
+    <mergeCell ref="G26:J31"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="M28:N29"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="L28:L29"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="I22:J22"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="I23:J23"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="I21:J21"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="D19:E19"/>
+    <mergeCell ref="I19:J19"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="I16:J16"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="I17:J17"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="I14:J14"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="I15:J15"/>
     <mergeCell ref="A13:C13"/>
     <mergeCell ref="D13:E13"/>
     <mergeCell ref="I13:J13"/>
@@ -1924,50 +1969,6 @@
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="D12:E12"/>
     <mergeCell ref="I12:J12"/>
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="I14:J14"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="I15:J15"/>
-    <mergeCell ref="A16:C16"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="I16:J16"/>
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="I17:J17"/>
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="I18:J18"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="D19:E19"/>
-    <mergeCell ref="I19:J19"/>
-    <mergeCell ref="A20:C20"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="A21:C21"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="I21:J21"/>
-    <mergeCell ref="A22:C22"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="I22:J22"/>
-    <mergeCell ref="A23:C23"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="I23:J23"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="M30:N30"/>
-    <mergeCell ref="B31:D31"/>
-    <mergeCell ref="A24:C24"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="I24:J24"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="B27:D27"/>
-    <mergeCell ref="B28:E28"/>
-    <mergeCell ref="G26:J31"/>
-    <mergeCell ref="A25:E25"/>
-    <mergeCell ref="M28:N29"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="L28:L29"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="5" scale="110" fitToWidth="0" orientation="landscape" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>